<commit_message>
get answers per query
</commit_message>
<xml_diff>
--- a/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
+++ b/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>query</t>
   </si>
@@ -25,6 +25,12 @@
     <t>top1_retrieved_chunk_mineru</t>
   </si>
   <si>
+    <t>answer_docling</t>
+  </si>
+  <si>
+    <t>answer_mineru</t>
+  </si>
+  <si>
     <t>Is detailed justification required when refining problems during the curation process?</t>
   </si>
   <si>
@@ -38,7 +44,28 @@
   </si>
   <si>
     <t xml:space="preserve">
-Result. Weshow the comparison results in Table D. Based on these results, in contrast to MM-UPD, we could not verify the efficacy of either the Option or Instruction approaches. This result reveals that the evaluation using MMMU fails to capture important findings of the effectiveness of these prompting approaches for UPD. Specifically, for expert-level problems, LMMs do not have accurate answers due to the lack of capability. Therefore, even if they choose an incorrect option when encountering...</t>
+Result. Weshow the comparison results in Table D. Based on these results, in contrast to MM-UPD, we could not verify the efficacy of either the Option or Instruction approaches. This result reveals that the evaluation using MMMU fails to capture important findings of the effectiveness of these prompting approaches for UPD. Specifically, for expert-level problems, LMMs do not have accurate answers due to the lack of capability. Therefore, even if they choose an incorrect option when encountering an unsolvable problem, this only indicates a lack of reasoning ability or knowledge and does not necessarily demonstrate a lack of refusal ability. Additionally, due to the very low overall performance, it becomes difficult to have meaningful discussions based on these minute differences in scores. Therefore, we exclude datasets with low Standard accuracy.
+## C Experimental Detail
+## C.1 Experimental Setup
+Computing Infrastructures. We conduct all our evaluations of open-source models on a single NVIDIA A100 (80GB) GPU.
+HyperParameters of LMM Inference. We set a temperature to 0 for all models during inference.
+## C.2 Detail of LLM-driven Methods
+In this section, we explain the details of the LLMdriven approaches in Sec. 5.3.
+Chain of Thought (CoT) Prompting. In this experiment, we investigate whether a widely used Zero-shot CoT (Kojima et al., 2022) is effective for UPD. We added the prompt 'Let's think step by step." at the end of the prompt and measured the performance.
+Self-reflection Self-reflection is a method that allows the model to reflect on its own responses (Kadavath et al., 2022). It has been shown that LLMs might have preliminary capabilities for judging and evaluating their own answers (Kadavath et al., 2022; Feng et al., 2024). In this experiment, we evaluate whether self-reflection is effective for UPD. We show the prompt for self-reflection in Table F. We prompt the LMM to self-reflect directly after its generated answer with the phrase 'The above answer is: 1. True 2. False,' following LLM protocols (Kadavath et al., 2022; Feng et al., 2024). For evaluation, if the LMM outputs '2. False," the response will be withdrawn. Otherwise, we use the original LMM's response for the evaluation.
+## D Additional Experiments
+We explore effective instruction-tuning recipes for solving UPD. To solve all kinds of UPD problems, we meticulously designed the data distribution for instruction tuning on Standard, AAD, IASD, and IVQD questions.
+Table C: Representative samples for removed questions for MM-IVQD construction
+| Ability                                     | Example of removed question                              |
+|---------------------------------------------|----------------------------------------------------------|
+| #3 Object Localization                      | How many dogs are in this picture?                       |
+| #15 Image Topic                             | Which one is the correct caption of this image?          |
+| #16 Image Emotion                           | Which mood does this image convey?                       |
+| #13 Structuralized Image-text Understanding | Which Python code can generate the content of the image? |
+| #14 Future Prediction                       | What will happen next?                                   |
+| #10 Identity Reasoning                      | What's the profession of the people in this picture?     |
+| #18 Image Style                             | Which style is represented in this image?                |
+</t>
   </si>
   <si>
     <t>Figure A: Relationship between OC-Dual accuracy and Dual accuracy.
@@ -55,29 +82,223 @@
 ## Gemini1.5Pro
 The function of the demonstrated object is to **play tennis**. Although none of the provided options are correct , the image clearly shows a tennis court.
 ## LLaVA-NeXT-34B
-The object in the image is a tennis racket, which is...</t>
+The object in the image is a tennis racket, which is used for playing tennis . The person in the image is holding the racket and appears to be in the middle of a tennis match or practice session.
+## InternVL2-40B
+The object in the image is a tennis racket, and it is being used to play tennis . Tennis is a sport that involves hitting a ball over a net with a racket, aiming to make the ball land within the opponent's court.
+- Q. What kind of human behavior does this picture describe?
+- A. A group of friends are rock climbing on a cliff face, using ropes and harnesses to ascend steep heights while feeling exhilarated by the challenge.
+- B. A musician is recording music in a studio, singing or playing instruments and perfecting tracks for an upcoming album.
+- C. A man is playing basketball at a court, dribbling, passing, and shooting hoops with precision and skill.
+## GPT-4o
+The picture describes a man standing in the rain with his arms outstretched and his face turned upwards , appearing to be experiencing a moment of emotional release or exhilaration. This does not match any of the provided options (A, B, or C).
+## Gemini1.5Pro
+None of the options provided describe the image . The image depicts a man standing in heavy rain with his arms outstretched and head tilted back .
+## LLaVA-NeXT-34B
+The image depicts a person with their arms outstretched , seemingly in a state of joy or exasperation, possibly after a swim or being in water.
+## InternVL2-40B
+The picture depicts a man standing in the rain with his arms outstretched .
+This behavior can be described as a form of emotional expression or a moment of connection with nature.
+&lt;!-- image --&gt;
+Figure J: Comparison of outputs of GPT-4o, Gemini1.5Pro, LLaVA-NeXT-34B, and InternVL2-40B. Green part is the description for the correct masked answer. Brown part points out the inability to solve the problem. Closedsource LMMs tend to point out both the correct answer and the fact that the problem cannot be solved, while open-source LMMs tend to only indicate the correct answer.
+&lt;!-- image --&gt;
+Figure K: Examples for AAD.
+&lt;!-- image --&gt;
+Figure L: Examples for AAD.
+&lt;!-- image --&gt;
+Figure M: Examples for IASD.
+&lt;!-- image --&gt;
+Figure N: Examples for IASD.
+&lt;!-- image --&gt;
+Figure O: Examples for IVQD.
+&lt;!-- image --&gt;
+1093
+Figure P: Examples for IVQD.
+&lt;!-- image --&gt;
+1093
+Table H: Full results for AAD in the base setting. We report Standard accuracy, AAD accuracy, and Dual accuracy.
+| #18   | 0.0 11.4 25.0 2.3 4.5 0.0 0.0 0.0 0.0 0.0 0.0 9.1 9.1 20.5 0.0 2.3 13.6 0.0 31.8 38.6 20.5 43.2                                                                                                                                                              | 0.0 22.7 31.8 4.5 6.8 0.0 0.0 2.3 0.0 0.0 0.0 11.4 11.4 27.3 0.0 2.3 18.2 0.0 34.1 43.2 25.0 45.5                                                                                                                                                                         | 18.2 22.7 50.0 6.8 43.2 6.8 27.3 25.0 34.1 43.2 47.7 27.3 45.5 59.1 27.3 47.7 70.5 47.7 77.3 72.7 68.2 75.0                                                                                                                                        |
+</t>
   </si>
   <si>
     <t xml:space="preserve">
-Clarification of the Semantics of the Options. We clarify the meaning of the options. Specifically, some questions in #6: Attribute Comparison have “Can’t judge”. “Can’t judge” means that “I can’t judge from the image since the image does not have enough information”. However, “Can’t judge” might be interpreted as “Since the given options are incorrect, can’t judge.” Therefore, we changed the option of “Can’t judge” to “Can’t judge from the image due to the lack of image information” to reduce...</t>
+Clarification of the Semantics of the Options. We clarify the meaning of the options. Specifically, some questions in #6: Attribute Comparison have “Can’t judge”. “Can’t judge” means that “I can’t judge from the image since the image does not have enough information”. However, “Can’t judge” might be interpreted as “Since the given options are incorrect, can’t judge.” Therefore, we changed the option of “Can’t judge” to “Can’t judge from the image due to the lack of image information” to reduce the ambiguity.
+After the above adaptation process, we construct MM-UPD Bench (MM-AAD, MM-IASD, MM-IVQD) as follows:
+## B.2 Construction of MM-AAD Bench
+When creating the MM-AAD Bench, we mask the correct options and remove all questions that originally have two options (which after removal would have only one option left). Also, we remove the questions whose answer is “both A,B, and C" and “all of these options are correct". To ensure no answer is present in the options, we also manually remove some questions with ambiguity where one of the remaining options is very similar to the masked correct option (e.g., Q. What can be the relationship of these people in this image? Masked Option: Friends, Similar remaining option: Colleagues). Our MM-AAD Bench has 820 AAD questions over 18 abilities. The distribution of questions for each ability is shown at the top of Table B.
+## B.3 Construction of MM-IASD Bench
+To create MM-IASD, we shuffle all questions and answer sets and pair each question with a random answer set. To further ensure the incompatibility, after the shuffling, we manually removed questions where the shuffled answer set was somehow compatible with the question (e.g., Q. Which of the following captions best describes this image? Correct answer: A person holding a bouquet of flowers, Similar shuffled option: Happiness). Our MM-IASD Bench has 919 IASD questions over 18 abilities. The distribution of questions for each ability is shown in the middle of Table B.
+## B.4 Construction of MM-IVQD Bench
+To create MM-IVQD Bench, we first exclude the questions that can be relevant to most images and then shuffle the original image-question pairs. In Table C, we show some representative examples of removed questions. For example, the question of “How many ..." can be compatible with any image, since the correct option of “None of the above" always exists for any image even when the image has no corresponding objects. For the question of “What’s the profession ...", we can interpret the profession from any kind of image (e.g., A beautifully captured image would suggest the profession of a photographer). In addition, we exclude the op tion “Can’t judge from the image due to the lack of image information.” because this option can be a correct answer for IVQD questions. Again, we conduct a manual check to guarantee the incompatibility of image-question pairs. Our MM-IVQD Bench has 356 IVQD questions over 12 abilities. The distribution of questions for each ability is shown in the bottom of Table B. Here, the lack of some ability (e.g.,#16 Image Emotion) indicates that there are many removed questions that can be applied to any image. Note that the small number of IVQD questions compared to AAD and IASD is due to our careful annotation and that even this number of questions is sufficient to show the performance difference between each LMM and method from our main experimental results.
+Here, one might wonder why we exclude questions rather than modify them. That is true that we can increase the number of questions by making the general question more specific. However, these question types are inherently less likely to encounter IVQD situations, and there is a concern that forcibly modifying the questions might lead to a divergence from real-world IVQD distribution. Moreover, incorporating numerous question types with low IVQD frequency could overshadow the significance of question types that are more likely to occur, thereby compromising the accurate assessment of IVQD performance. Therefore, we chose to exclude these questions rather than modify them.
+## B.5 Manual Curation Procedure
+The dataset curation is carried out by four annotators from the authors. To improve the efficiency of collaborative curation and ensure consistency in quality, we first transcribed the image-question pairs from MMBench into an online editing tool (i.e., Google Docs) and conducted the curation process directly within the platform. To enhance the consistency, each question was independently reviewed by two annotators. Finally, the lead author verified the validity of all curation. If a problem needed to be refined, the reason was recorded in detail as a comment. For example, in the case of IVQD, which required the most careful curation, one annotator would leave a comment on points such as “The reason the image relates to the question is..." or “If we change this image into ..., the irrelevance is guaranteed.". If another annotator agreed with the comment, the problem was refined. In cases where the other annotator disagreed, all four annotators engaged in discussions to reach a consensus.
+We consider that collaborative tools such as Google Docs, double-checking by two annotators, and detailed justifications with collective decisions ensure curation consistency.
+## B.6 Validity of UPD Benchmark on More Complex Datasets
+The reason for the exclusion of the recent challenging dataset (e.g., MMMU (Yue et al., 2024a)) for our UPD benchmark is that the evaluation significantly deviates from the aspect of reliability and potentially causes us to miss important findings. To verify this, we conducted experiments with MMMU in the AAD setting.
+</t>
   </si>
   <si>
     <t xml:space="preserve">
 Table 1: Comparison results of the overall Dual accuracy for the base setting, additional-option setting, and additional-instruction setting. The “Orig” (Original Standard) value is the upper bound of Dual accuracy. The results show that the difference between each Dual accuracy and the Original Standard is clear and most open-source LMMs have significantly low scores.</t>
   </si>
   <si>
-    <t>ail
+    <t xml:space="preserve">ail
 ## C.1 Experimental Setup
 Computing Infrastructures. We conduct all our evaluations of open-source models on a single NVIDIA A100 (80GB) GPU.
 HyperParameters of LMM Inference. We set a temperature to 0 for all models during inference.
 ## C.2 Detail of LLM-driven Methods
 In this section, we explain the details of the LLMdriven approaches in Sec. 5.3.
-Chain of Thought (CoT) Prompting. In this experiment, we investigate whether a widely used Zero-shot CoT (Kojima et al., 2022) is effectiv...</t>
+Chain of Thought (CoT) Prompting. In this experiment, we investigate whether a widely used Zero-shot CoT (Kojima et al., 2022) is effective for UPD. We added the prompt “Let’s think step by step." at the end of the prompt and measured the performance.
+Self-reflection Self-reflection is a method that allows the model to reflect on its own responses (Kadavath et al., 2022). It has been shown that LLMs might have preliminary capabilities for judging and evaluating their own answers (Kadavath et al., 2022; Feng et al., 2024). In this experiment, we evaluate whether self-reflection is effective for UPD. We show the prompt for self-reflection in Table F. We prompt the LMM to self-reflect directly after its generated answer with the phrase “The above answer is: 1. True 2. False,” following LLM protocols (Kadavath et al., 2022; Feng et al., 2024). For evaluation, if the LMM outputs “2. False," the response will be withdrawn. Otherwise, we use the original LMM’s response for the evaluation.
+## D Additional Experiments
+We explore effective instruction-tuning recipes for solving UPD. To solve all kinds of UPD problems, we meticulously designed the data distribution for instruction tuning on Standard, AAD, IASD, and IVQD questions.
+</t>
   </si>
   <si>
     <t xml:space="preserve">
 Marah Abdin, Sam Ade Jacobs, Ammar Ahmad Awan, Jyoti Aneja, Ahmed Awadallah, Hany Awadalla, Nguyen Bach, Amit Bahree, Arash Bakhtiari, Harkirat Behl, et al. 2024. Phi-3 technical report: A highly capable language model locally on your phone. arXiv preprint arXiv:2404.14219.
-Josh Achiam, Steven Adler, Sandhini Agarwal, Lama Ahmad, Ilge Akkaya, Florencia Leoni Aleman, Diogo Almeida, Janko Altenschmidt, Sam Altman, Shyamal Anadkat, et al. 2023. Gpt-4 technical report. arXiv preprint arXiv:2303.0...</t>
+Josh Achiam, Steven Adler, Sandhini Agarwal, Lama Ahmad, Ilge Akkaya, Florencia Leoni Aleman, Diogo Almeida, Janko Altenschmidt, Sam Altman, Shyamal Anadkat, et al. 2023. Gpt-4 technical report. arXiv preprint arXiv:2303.08774.
+Syeda Nahida Akter, Sangwu Lee, Yingshan Chang, Yonatan Bisk, and Eric Nyberg. 2024. Visreas: Complex visual reasoning with unanswerable questions. In ACL Findings.
+Jean-Baptiste Alayrac, Jeff Donahue, Pauline Luc, Antoine Miech, Iain Barr, Yana Hasson, Karel Lenc, Arthur Mensch, Katherine Millican, Malcolm Reynolds, et al. 2022. Flamingo: a visual language model for few-shot learning. In NeurIPS.
+Dario Amodei, Chris Olah, Jacob Steinhardt, Paul Christiano, John Schulman, and Dan Mané. 2016. Concrete problems in ai safety. arXiv preprint arXiv:1606.06565.
+Stanislaw Antol, Aishwarya Agrawal, Jiasen Lu, Margaret Mitchell, Dhruv Batra, C Lawrence Zitnick, and Devi Parikh. 2015. Vqa: Visual question answering. In ICCV.
+Anas Awadalla, Irena Gao, Josh Gardner, Jack Hessel, Yusuf Hanafy, Wanrong Zhu, Kalyani Marathe, Yonatan Bitton, Samir Gadre, Shiori Sagawa, et al. 2023. Openflamingo: An open-source framework for training large autoregressive vision-language models. arXiv preprint arXiv:2308.01390.
+Nilavra Bhattacharya, Qing Li, and Danna Gurari. 2019. Why does a visual question have different answers? In ICCV.
+Qingxing Cao, Junhao Cheng, Xiaodan Liang, and Liang Lin. 2024. Visdiahalbench: A visual dialogue benchmark for diagnosing hallucination in large vision-language models. In ACL.
+Lichang Chen, Shiyang Li, Jun Yan, Hai Wang, Kalpa Gunaratna, Vikas Yadav, Zheng Tang, Vijay Srinivasan, Tianyi Zhou, Heng Huang, et al. 2024a. Alpagasus: Training a better alpaca with fewer data. In ICLR.
+Lin Chen, Jinsong Li, Xiaoyi Dong, Pan Zhang, Yuhang Zang, Zehui Chen, Haodong Duan, Jiaqi Wang, Yu Qiao, Dahua Lin, et al. 2024b. Are we on the right way for evaluating large vision-language models? In NeurIPS.
+Yen-Chun Chen, Linjie Li, Licheng Yu, Ahmed El Kholy, Faisal Ahmed, Zhe Gan, Yu Cheng, and Jingjing Liu. 2020. Uniter: Universal image-text representation learning. In ECCV.
+Zhe Chen, Weiyun Wang, Hao Tian, Shenglong Ye, Zhangwei Gao, Erfei Cui, Wenwen Tong, Kongzhi Hu, Jiapeng Luo, Zheng Ma, et al. 2024c. How far are we to gpt-4v? closing the gap to commercial multimodal models with open-source suites. arXiv preprint arXiv:2404.16821.
+Wei-Lin Chiang, Zhuohan Li, Zi Lin, Ying Sheng, Zhanghao Wu, Hao Zhang, Lianmin Zheng, Siyuan Zhuang, Yonghao Zhuang, Joseph E. Gonzalez, Ion Stoica, and Eric P. Xing. 2023. Vicuna: An opensource chatbot impressing gpt-4 with 90%\* chatgpt quality.
+Eunsol Choi, He He, Mohit Iyyer, Mark Yatskar, Wentau Yih, Yejin Choi, Percy Liang, and Luke Zettlemoyer. 2018. Quac: Question answering in context. In EMNLP.
+Hyung Won Chung, Le Hou, Shayne Longpre, Barret Zoph, Yi Tay, William Fedus, Yunxuan Li, Xuezhi Wang, Mostafa Dehghani, Siddhartha Brahma, et al. 2024. Scaling instruction-finetuned language models. JMLR, 25(70):1–53.
+Chenhang Cui, Yiyang Zhou, Xinyu Yang, Shirley Wu, Linjun Zhang, James Zou, and Huaxiu Yao. 2023. Holistic analysis of hallucination in gpt-4v (ision):
+Bias and interference challenges. arXiv preprint arXiv:2311.03287.
+Wenliang Dai, Junnan Li, Dongxu Li, Anthony Tiong, Junqi Zhao, Weisheng Wang, Boyang Li, Pascale Fung, and Steven Hoi. 2023. InstructBLIP: Towards general-purpose vision-language models with instruction tuning. In NeurIPS.
+Ernest Davis. 2020. Unanswerable questions about images and texts. Frontiers in Artificial Intelligence, 3:51.
+Xuefeng Du, Zhaoning Wang, Mu Cai, and Yixuan Li. 2022. Vos: Learning what you don’t know by virtual outlier synthesis. In ICLR.
+Sepideh Esmaeilpour, Bing Liu, Eric Robertson, and Lei Shu. 2022. Zero-shot out-of-distribution detection based on the pretrained model clip. In AAAI.
+Alessandro Favero, Luca Zancato, Matthew Trager, Siddharth Choudhary, Pramuditha Perera, Alessandro Achille, Ashwin Swaminathan, and Stefano Soatto. 2024. Multi-modal hallucination control by visual information grounding. In CVPR.
+Shangbin Feng, Weijia Shi, Yike Wang, Wenxuan Ding, Vidhisha Balachandran, and Yulia Tsvetkov. 2024. Don’t hallucinate, abstain: Identifying llm knowledge gaps via multi-llm collaboration. In ACL.
+Xingyu Fu, Yushi Hu, Bangzheng Li, Yu Feng, Haoyu Wang, Xudong Lin, Dan Roth, Noah A Smith, Wei-Chiu Ma, and Ranjay Krishna. 2024. Blink: Multimodal large language models can see but not perceive. In ECCV.
+Peng Gao, Jiaming Han, Renrui Zhang, Ziyi Lin, Shijie Geng, Aojun Zhou, Wei Zhang, Pan Lu, Conghui He, Xiangyu Yue, et al. 2023. Llama-adapter v2: Parameter-efficient visual instruction model. arXiv preprint arXiv:2304.15010.
+Yash Goyal, Tejas Khot, Douglas Summers-Stay, Dhruv Batra, and Devi Parikh. 2017. Making the v in vqa matter: Elevating the role of image understanding in visual question answering. In CVPR.
+Tianrui Guan, Fuxiao Liu, Xiyang Wu, Ruiqi Xian, Zongxia Li, Xiaoyu Liu, Xijun Wang, Lichang Chen, Furong Huang, Yaser Yacoob, Dinesh Manocha, and Tianyi Zhou. 2024. Hallusionbench: An advanced diagnostic suite for entangled language hallucination &amp; visual illusion in large vision-language models. In CVPR.
+Anisha Gunjal, Jihan Yin, and Erhan Bas. 2024. Detecting and preventing hallucinations in large vision language models. In AAAI.
+Yanyang Guo, Fangkai Jiao, Zhiqi Shen, Liqiang Nie, and Mohan Kankanhalli. 2024. Unk-vqa: A dataset and a probe into the abstention ability of multi-modal large models. TPAMI.
+Danna Gurari, Qing Li, Abigale J Stangl, Anhong Guo, Chi Lin, Kristen Grauman, Jiebo Luo, and Jeffrey P Bigham. 2018. Vizwiz grand challenge: Answering visual questions from blind people. In CVPR.
+Dan Hendrycks, Nicholas Carlini, John Schulman, and Jacob Steinhardt. 2021. Unsolved problems in ml safety. arXiv preprint arXiv:2109.13916.
+Dan Hendrycks and Kevin Gimpel. 2017. A baseline for detecting misclassified and out-of-distribution examples in neural networks. In ICLR.
+Dan Hendrycks and Mantas Mazeika. 2022. Xrisk analysis for ai research. arXiv preprint arXiv:2206.05862.
+Wenyi Hong, Weihan Wang, Ming Ding, Wenmeng Yu, Qingsong Lv, Yan Wang, Yean Cheng, Shiyu Huang, Junhui Ji, Zhao Xue, et al. 2024. Cogvlm2: Visual language models for image and video understanding. arXiv preprint arXiv:2408.16500.
+Edward J Hu, Yelong Shen, Phillip Wallis, Zeyuan Allen-Zhu, Yuanzhi Li, Shean Wang, Lu Wang, and Weizhu Chen. 2022. LoRA: Low-rank adaptation of large language models. In ICLR.
+Wenbo Hu, Jia-Chen Gu, Zi-Yi Dou, Mohsen Fayyaz, Pan Lu, Kai-Wei Chang, and Nanyun Peng. 2025. Mrag-bench: Vision-centric evaluation for retrievalaugmented multimodal models. In ICLR.
+Qidong Huang, Xiaoyi Dong, Pan Zhang, Bin Wang, Conghui He, Jiaqi Wang, Dahua Lin, Weiming Zhang, and Nenghai Yu. 2024. Opera: Alleviating hallucination in multi-modal large language models via over-trust penalty and retrospection-allocation. In CVPR.
+Drew A Hudson and Christopher D Manning. 2019. Gqa: A new dataset for real-world visual reasoning and compositional question answering. In CVPR.
+Aaron Hurst, Adam Lerer, Adam P Goucher, Adam Perelman, Aditya Ramesh, Aidan Clark, AJ Ostrow, Akila Welihinda, Alan Hayes, Alec Radford, et al. 2024. Gpt-4o system card. arXiv preprint arXiv:2410.21276.
+Chaoya Jiang, Haiyang Xu, Mengfan Dong, Jiaxing Chen, Wei Ye, Ming Yan, Qinghao Ye, Ji Zhang, Fei Huang, and Shikun Zhang. 2024. Hallucination augmented contrastive learning for multimodal large language model. In CVPR.
+Saurav Kadavath, Tom Conerly, Amanda Askell, Tom Henighan, Dawn Drain, Ethan Perez, Nicholas Schiefer, Zac Hatfield-Dodds, Nova DasSarma, Eli Tran-Johnson, et al. 2022. Language models (mostly) know what they know. arXiv preprint arXiv:2207.05221.
+Takeshi Kojima, Shixiang Shane Gu, Machel Reid, Yutaka Matsuo, and Yusuke Iwasawa. 2022. Large language models are zero-shot reasoners. In NeurIPS.
+Hugo Laurençon, Andrés Marafioti, Victor Sanh, and Léo Tronchon. 2024a. Building and better understanding vision-language models: insights and future directions. arXiv preprint arXiv:2408.12637.
+Hugo Laurençon, Léo Tronchon, Matthieu Cord, and Victor Sanh. 2024b. What matters when building vision-language models? In NeurIPS.
+Bo Li, Yuanhan Zhang, Liangyu Chen, Jinghao Wang, Jingkang Yang, and Ziwei Liu. 2023a. Otter: A multi-modal model with in-context instruction tuning. arXiv preprint arXiv:2305.03726.
+Bo Li, Yuanhan Zhang, Dong Guo, Renrui Zhang, Feng Li, Hao Zhang, Kaichen Zhang, Yanwei Li, Ziwei Liu, and Chunyuan Li. 2024a. Llavaonevision: Easy visual task transfer. arXiv preprint arXiv:2408.03326.
+Bohao Li, Rui Wang, Guangzhi Wang, Yuying Ge, Yixiao Ge, and Ying Shan. 2024b. Seed-bench: Benchmarking multimodal llms with generative comprehension. In CVPR.
+Feng Li, Renrui Zhang, Hao Zhang, Yuanhan Zhang, Bo Li, Wei Li, Zejun Ma, and Chunyuan Li. 2025. Llava-next-interleave: Tackling multi-image, video, and 3d in large multimodal models. In ICLR.
+Xiujun Li, Xi Yin, Chunyuan Li, Pengchuan Zhang, Xiaowei Hu, Lei Zhang, Lijuan Wang, Houdong Hu, Li Dong, Furu Wei, et al. 2020. Oscar: Objectsemantics aligned pre-training for vision-language tasks. In ECCV.
+Yifan Li, Yifan Du, Kun Zhou, Jinpeng Wang, Wayne Xin Zhao, and Ji-Rong Wen. 2023b. Evaluating object hallucination in large vision-language models. In EMNLP.
+Shiyu Liang, Yixuan Li, and Rayadurgam Srikant. 2018. Enhancing the reliability of out-of-distribution image detection in neural networks. In ICLR.
+Ji Lin, Hongxu Yin, Wei Ping, Pavlo Molchanov, Mohammad Shoeybi, and Song Han. 2024. Vila: On pre-training for visual language models. In CVPR.
+Tsung-Yi Lin, Michael Maire, Serge Belongie, James Hays, Pietro Perona, Deva Ramanan, Piotr Dollár, and C Lawrence Zitnick. 2014. Microsoft coco: Common objects in context. In ECCV.
+Fuxiao Liu, Kevin Lin, Linjie Li, Jianfeng Wang, Yaser Yacoob, and Lijuan Wang. 2024a. Aligning large multi-modal model with robust instruction tuning. In ICLR.
+Fuxiao Liu, Hao Tan, and Chris Tensmeyer. 2024b. Documentclip: Linking figures and main body text in reflowed documents. In ICPRAI.
+Haotian Liu, Chunyuan Li, Yuheng Li, and Yong Jae Lee. 2024c. Improved baselines with visual instruction tuning. In CVPR.
+Haotian Liu, Chunyuan Li, Yuheng Li, Bo Li, Yuanhan Zhang, Sheng Shen, and Yong Jae Lee. 2024d. Llavanext: Improved reasoning, ocr, and world knowledge.
+Haotian Liu, Chunyuan Li, Qingyang Wu, and Yong Jae Lee. 2023. Visual instruction tuning. In NeurIPS.
+Yuan Liu, Haodong Duan, Yuanhan Zhang, Bo Li, Songyang Zhang, Wangbo Zhao, Yike Yuan, Jiaqi Wang, Conghui He, Ziwei Liu, et al. 2024e. Mmbench: Is your multi-modal model an all-around player? In ECCV.
+Pan Lu, Hritik Bansal, Tony Xia, Jiacheng Liu, Chunyuan Li, Hannaneh Hajishirzi, Hao Cheng, Kai-Wei Chang, Michel Galley, and Jianfeng Gao. 2024. Mathvista: Evaluating mathematical reasoning of foundation models in visual contexts. In ICLR.
+Kenneth Marino, Mohammad Rastegari, Ali Farhadi, and Roozbeh Mottaghi. 2019. Ok-vqa: A visual question answering benchmark requiring external knowledge. In CVPR.
+Yifei Ming, Ziyang Cai, Jiuxiang Gu, Yiyou Sun, Wei Li, and Yixuan Li. 2022a. Delving into out-ofdistribution detection with vision-language representations. In NeurIPS.
+Yifei Ming, Hang Yin, and Yixuan Li. 2022b. On the impact of spurious correlation for out-of-distribution detection. In AAAI.
+Atsuyuki Miyai, Jingkang Yang, Jingyang Zhang, Yifei Ming, Yueqian Lin, Qing Yu, Go Irie, Shafiq Joty, Yixuan Li, Hai Li, et al. 2024. Generalized out-of-distribution detection and beyond in vision language model era: A survey. arXiv preprint arXiv:2407.21794.
+Atsuyuki Miyai, Qing Yu, Go Irie, and Kiyoharu Aizawa. 2023a. Can pre-trained networks detect familiar out-of-distribution data? arXiv preprint arXiv:2310.00847.
+Atsuyuki Miyai, Qing Yu, Go Irie, and Kiyoharu Aizawa. 2023b. Locoop: Few-shot out-ofdistribution detection via prompt learning. In NeurIPS.
+Sina Mohseni, Haotao Wang, Chaowei Xiao, Zhiding Yu, Zhangyang Wang, and Jay Yadawa. 2022. Taxonomy of machine learning safety: A survey and primer. ACM Computing Surveys, 55(8):1–38.
+Masoud Monajatipoor, Liunian Harold Li, Mozhdeh Rouhsedaghat, Lin F Yang, and Kai-Wei Chang. 2024. Metavl: Transferring in-context learning ability from language models to vision-language models. In ACL.
+OpenAI. 2023. Gpt-4v(ision) system card.
+OpenAI. 2024. gpt-4o mini: advancing cost-efficient intelligence.
+Dongmin Park, Zhaofang Qian, Guangxing Han, and Ser-Nam Lim. 2024. Mitigating dialogue hallucination for large multi-modal models via adversarial instruction tuning. arXiv preprint arXiv:2403.10492.
+Pranav Rajpurkar, Robin Jia, and Percy Liang. 2018. Know what you don’t know: Unanswerable questions for squad. In ACL.
+Siva Reddy, Danqi Chen, and Christopher D Manning. 2019. Coqa: A conversational question answering challenge. TACL, 7:249–266.
+Machel Reid, Nikolay Savinov, Denis Teplyashin, Dmitry Lepikhin, Timothy Lillicrap, Jean-baptiste Alayrac, Radu Soricut, Angeliki Lazaridou, Orhan Firat, Julian Schrittwieser, et al. 2024. Gemini 1.5: Unlocking multimodal understanding across millions of tokens of context. arXiv preprint arXiv:2403.05530.
+Joshua Robinson, Christopher Rytting, and David Wingate. 2023. Leveraging large language models for multiple choice question answering. In ICLR.
+Anna Rohrbach, Lisa Anne Hendricks, Kaylee Burns, Trevor Darrell, and Kate Saenko. 2018. Object hallucination in image captioning. In EMNLP.
+Dustin Schwenk, Apoorv Khandelwal, Christopher Clark, Kenneth Marino, and Roozbeh Mottaghi. 2022. A-okvqa: A benchmark for visual question answering using world knowledge. In ECCV.
+Elior Sulem, Jamaal Hay, and Dan Roth. 2022. Yes, no or IDK: The challenge of unanswerable yes/no questions. In NAACL.
+Zhiqing Sun, Sheng Shen, Shengcao Cao, Haotian Liu, Chunyuan Li, Yikang Shen, Chuang Gan, Liang-Yan Gui, Yu-Xiong Wang, Yiming Yang, et al. 2024. Aligning large multimodal models with factually augmented rlhf. In ACL Findings.
+Gemini Team, Rohan Anil, Sebastian Borgeaud, Yonghui Wu, Jean-Baptiste Alayrac, Jiahui Yu, Radu Soricut, Johan Schalkwyk, Andrew M Dai, Anja Hauth, et al. 2023. Gemini: a family of highly capable multimodal models. arXiv preprint arXiv:2312.11805.
+Qwen Team. 2025. Qwen2.5-vl.
+Hugo Touvron, Thibaut Lavril, Gautier Izacard, Xavier Martinet, Marie-Anne Lachaux, Timothée Lacroix, Baptiste Rozière, Naman Goyal, Eric Hambro, Faisal Azhar, et al. 2023. Llama: Open and efficient foundation language models. arXiv preprint arXiv:2302.13971.
+Haochun Wang, Sendong Zhao, Zewen Qiang, Bing Qin, and Ting Liu. 2025. Llms may perform mcqa by selecting the least incorrect option. In COLING.
+Haoran Wang, Weitang Liu, Alex Bocchieri, and Yixuan Li. 2021. Can multi-label classification networks know what they don’t know? In NeurIPS.
+Hualiang Wang, Yi Li, Huifeng Yao, and Xiaomeng Li. 2023a. Clipn for zero-shot ood detection: Teaching clip to say no. In ICCV.
+Junyang Wang, Yiyang Zhou, Guohai Xu, Pengcheng Shi, Chenlin Zhao, Haiyang Xu, Qinghao Ye, Ming Yan, Ji Zhang, Jihua Zhu, et al. 2023b. Evaluation and analysis of hallucination in large vision-language models. arXiv preprint arXiv:2308.15126.
+Peiyi Wang, Lei Li, Liang Chen, Zefan Cai, Dawei Zhu, Binghuai Lin, Yunbo Cao, Qi Liu, Tianyu Liu, and Zhifang Sui. 2024a. Large language models are not fair evaluators. In ACL.
+Peng Wang, Shuai Bai, Sinan Tan, Shijie Wang, Zhihao Fan, Jinze Bai, Keqin Chen, Xuejing Liu, Jialin Wang, Wenbin Ge, et al. 2024b. Qwen2-vl: Enhancing vision-language model’s perception of the world at any resolution. arXiv preprint arXiv:2409.12191.
+Weihan Wang, Qingsong Lv, Wenmeng Yu, Wenyi Hong, Ji Qi, Yan Wang, Junhui Ji, Zhuoyi Yang, Lei Zhao, Xixuan Song, et al. 2023c. Cogvlm: Visual expert for pretrained language models. arXiv preprint arXiv:2311.03079.
+Xintong Wang, Jingheng Pan, Liang Ding, and Chris Biemann. 2024c. Mitigating hallucinations in large vision-language models with instruction contrastive decoding. In ACL Findings.
+Jerry Wei, Jason Wei, Yi Tay, Dustin Tran, Albert Webson, Yifeng Lu, Xinyun Chen, Hanxiao Liu, Da Huang, Denny Zhou, et al. 2023. Larger language models do in-context learning differently. arXiv preprint arXiv:2303.03846.
+Spencer Whitehead, Suzanne Petryk, Vedaad Shakib, Joseph Gonzalez, Trevor Darrell, Anna Rohrbach, and Marcus Rohrbach. 2022. Reliable visual question answering: Abstain rather than answer incorrectly. In ECCV.
+Le Xue, Manli Shu, Anas Awadalla, Jun Wang, An Yan, Senthil Purushwalkam, Honglu Zhou, Viraj Prabhu, Yutong Dai, Michael S Ryoo, et al. 2024. xgen-mm (blip-3): A family of open large multimodal models. arXiv preprint arXiv:2408.08872.
+An Yang, Baosong Yang, Binyuan Hui, Bo Zheng, Bowen Yu, Chang Zhou, Chengpeng Li, Chengyuan Li, Dayiheng Liu, Fei Huang, et al. 2024a. Qwen2 technical report. arXiv preprint arXiv:2407.10671.
+Jingkang Yang, Pengyun Wang, Dejian Zou, Zitang Zhou, Kunyuan Ding, Wenxuan Peng, Haoqi Wang, Guangyao Chen, Bo Li, Yiyou Sun, Xuefeng Du, Kaiyang Zhou, Wayne Zhang, Dan Hendrycks, Yixuan Li, and Ziwei Liu. 2022. Openood: Benchmarking generalized out-of-distribution detection. In NeurIPS Datasets and Benchmarks Track.
+Jingkang Yang, Kaiyang Zhou, Yixuan Li, and Ziwei Liu. 2024b. Generalized out-of-distribution detection: A survey. International Journal of Computer Vision, 132(12):5635–5662.
+Jingkang Yang, Kaiyang Zhou, and Ziwei Liu. 2023. Full-spectrum out-of-distribution detection. IJCV, 131(10):2607–2622.
+Qinghao Ye, Haiyang Xu, Guohai Xu, Jiabo Ye, Ming Yan, Yiyang Zhou, Junyang Wang, Anwen Hu, Pengcheng Shi, Yaya Shi, et al. 2023. mplug-owl: Modularization empowers large language models with multimodality. arXiv preprint arXiv:2304.14178.
+Qinghao Ye, Haiyang Xu, Jiabo Ye, Ming Yan, Anwen Hu, Haowei Liu, Qi Qian, Ji Zhang, and Fei Huang. 2024. mplug-owl2: Revolutionizing multi-modal large language model with modality collaboration. In CVPR.
+Shukang Yin, Chaoyou Fu, Sirui Zhao, Tong Xu, Hao Wang, Dianbo Sui, Yunhang Shen, Ke Li, Xing Sun, and Enhong Chen. 2024. Woodpecker: Hallucination correction for multimodal large language models. Science China Information Sciences.
+Qing Yu and Kiyoharu Aizawa. 2019. Unsupervised out-of-distribution detection by maximum classifier discrepancy. In ICCV.
+Weihao Yu, Zhengyuan Yang, Linjie Li, Jianfeng Wang, Kevin Lin, Zicheng Liu, Xinchao Wang, and Lijuan Wang. 2024. Mm-vet: Evaluating large multimodal models for integrated capabilities. In ICML.
+Xiang Yue, Yuansheng Ni, Kai Zhang, Tianyu Zheng, Ruoqi Liu, Ge Zhang, Samuel Stevens, Dongfu Jiang, Weiming Ren, Yuxuan Sun, et al. 2024a. Mmmu: A massive multi-discipline multimodal understanding and reasoning benchmark for expert agi. In CVPR.
+Xiang Yue, Tianyu Zheng, Yuansheng Ni, Yubo Wang, Kai Zhang, Shengbang Tong, Yuxuan Sun, Ming Yin, Botao Yu, Ge Zhang, et al. 2024b. Mmmu-pro: A more robust multi-discipline multimodal understanding benchmark. arXiv preprint arXiv:2409.02813.
+Jingyang Zhang, Jingkang Yang, Pengyun Wang, Haoqi Wang, Yueqian Lin, Haoran Zhang, Yiyou Sun, Xuefeng Du, Kaiyang Zhou, Wayne Zhang, et al. 2024a. Openood v1. 5: Enhanced benchmark for out-ofdistribution detection. DMLR.
+Pan Zhang, Xiaoyi Dong, Yuhang Zang, Yuhang Cao, Rui Qian, Lin Chen, Qipeng Guo, Haodong Duan, Bin Wang, Linke Ouyang, Songyang Zhang, Wenwei Zhang, Yining Li, Yang Gao, Peng Sun, Xinyue Zhang, Wei Li, Jingwen Li, Wenhai Wang, Hang Yan, Conghui He, Xingcheng Zhang, Kai Chen, Jifeng Dai, Yu Qiao, Dahua Lin, and Jiaqi Wang. 2024b. Internlm-xcomposer-2.5: A versatile large vision language model supporting long-contextual input and output. arXiv preprint arXiv:2407.03320.
+Pengchuan Zhang, Xiujun Li, Xiaowei Hu, Jianwei Yang, Lei Zhang, Lijuan Wang, Yejin Choi, and Jianfeng Gao. 2021. Vinvl: Revisiting visual representations in vision-language models. In CVPR.
+Renrui Zhang, Jiaming Han, Aojun Zhou, Xiangfei Hu, Shilin Yan, Pan Lu, Hongsheng Li, Peng Gao, and Yu Qiao. 2024c. Llama-adapter: Efficient fine-tuning of language models with zero-init attention. In ICLR.
+Renrui Zhang, Dongzhi Jiang, Yichi Zhang, Haokun Lin, Ziyu Guo, Pengshuo Qiu, Aojun Zhou, Pan Lu, Kai-Wei Chang, Peng Gao, et al. 2024d. Mathverse: Does your multi-modal llm truly see the diagrams in visual math problems? In ECCV.
+Bo Zhao, Boya Wu, and Tiejun Huang. 2023. Svit: Scaling up visual instruction tuning. arXiv preprint arXiv:2307.04087.
+Haozhe Zhao, Zefan Cai, Shuzheng Si, Xiaojian Ma, Kaikai An, Liang Chen, Zixuan Liu, Sheng Wang, Wenjuan Han, and Baobao Chang. 2024. Mmicl: Empowering vision-language model with multi-modal in-context learning. In ICLR.
+Chujie Zheng, Hao Zhou, Fandong Meng, Jie Zhou, and Minlie Huang. 2025. Large language models are not robust multiple choice selectors. In ICLR.
+Luowei Zhou, Hamid Palangi, Lei Zhang, Houdong Hu, Jason Corso, and Jianfeng Gao. 2020. Unified visionlanguage pre-training for image captioning and vqa. In AAAI.
+Yiyang Zhou, Chenhang Cui, Jaehong Yoon, Linjun Zhang, Zhun Deng, Chelsea Finn, Mohit Bansal, and Huaxiu Yao. 2024. Analyzing and mitigating object hallucination in large vision-language models. In ICLR.
+Deyao Zhu, Jun Chen, Xiaoqian Shen, Xiang Li, and Mohamed Elhoseiny. 2024. Minigpt-4: Enhancing vision-language understanding with advanced large language models. In ICLR.
+## Appendix
+## A Additional Related Work
+Large Multimodal Model (LMM). Recent advancements in multimodal models have been driven by innovative training methods (Chen et al., 2020; Zhou et al., 2020; Zhang et al., 2021; Li et al., 2020; Alayrac et al., 2022; Awadalla et al., 2023). Following the success of large language models (LLMs), many LMMs have been developed with improved instruction-following capabilities (Liu et al., 2023, 2024c,d; Li et al., 2024a; Dai et al., 2023; Zhu et al., 2024; Zhang et al., 2024c; Gao et al., 2023; Ye et al., 2023, 2024; Zhao et al., 2023; Li et al., 2023a; Monajatipoor et al., 2024; Zhao et al., 2024; Li et al., 2025; Lin et al., 2024; Zhang et al., 2024b). Additionally, closed-source LMMs like GPT-4V (Achiam et al., 2023), GPT-4o (Hurst et al., 2024), and Gemini (Team et al., 2023) have exhibited strong performance across various visionlanguage tasks. However, a significant challenge remains in accurately evaluating the trustworthiness of these LMMs, highlighting the need for more robust and comprehensive benchmarks.
+LMM Benchmarks. As multi-modal pretraining and instruction tuning has gained prominence, the previous standard evaluation benchmarks e.g., VQA (Antol et al., 2015; Goyal et al., 2017), OK-VQA (Marino et al., 2019), COCO (Lin et al., 2014), and GQA (Hudson and Manning, 2019) become insufficient (Yue et al., 2024a,b). To more comprehensively assess the capabilities of LMMs, recent efforts have introduced benchmarks such as SEED (Li et al., 2024b), LLaVA-Bench (Liu et al., 2023), MMBench (Liu et al., 2024e), MM-Vet (Yu et al., 2024), MathVista (Lu et al., 2024), Mathverse (Zhang et al., 2024d), MMStar (Chen et al., 2024b), BLINK (Fu et al., 2024), MMMU (Yue et al., 2024a), and MMMU-Pro (Yue et al., 2024b) have emerged and become common benchmarks for evaluating LMMs (Li et al., 2024a). Among these, MMBench provides evaluations across a broad range of fine-grained abilities, which is highly important for assessing UPD. Therefore, by adopting MMBench, we can (i) evaluate performance across a wider range of tasks compared to similar recent works (Guo et al., 2024; Akter et al., 2024; Cao et al., 2024) that adopt conventional benchmarks (Lin et al., 2014; Goyal et al., 2017), and (ii) emphasize the challenge of UPD by comparing standard MMBench performance with
+UPD performance.
+Model Hallucinations. In LMMs, “hallucination” typically refers to situations where the generated responses contain information that is inconsistent in the visual content (Rohrbach et al., 2018; Wang et al., 2023b; Zhou et al., 2024; Guan et al., 2024; Sun et al., 2024; Cui et al., 2023; Jiang et al., 2024). Recent LMMs, such as LLaVA (Chung et al., 2024; Liu et al., 2024c), have also encountered the challenge of hallucination (Jiang et al., 2024). To evaluate hallucination in LMMs, various benchmarks, POPE (Li et al., 2023b), M-HalDetect (Gunjal et al., 2024), GAVIE (Liu et al., 2024a), Hallusion-Bench (Guan et al., 2024), and Bingo (Cui et al., 2023) have been proposed. Hallucination evaluation and detection (Li et al., 2023b; Wang et al., 2023b; Liu et al., 2024a), and hallucination mitigation (Yin et al., 2024; Zhou et al., 2024; Gunjal et al., 2024; Liu et al., 2024a; Favero et al., 2024; Huang et al., 2024; Park et al., 2024; Wang et al., 2024c) have also been explored. These existing studies deal with a wide range of hallucination issues. Unlike previous works, we address the hallucination issues where the LMM produces incorrect responses when presented with unsolvable problems. Only a few very recent works have addressed this type of hallucination (Guo et al., 2024; Akter et al., 2024; Cao et al., 2024). However, they do not assess the robustness of LMMs for common MCQA.
+AI Safety. A reliable visual recognition system should not only produce accurate predictions on known context but also detect unknown examples (Amodei et al., 2016; Mohseni et al., 2022; Hendrycks et al., 2021; Hendrycks and Mazeika, 2022). The representative research field to address this safety aspect is out-of-distribution (OOD) detection (Hendrycks and Gimpel, 2017; Liang et al., 2018; Yang et al., 2024b, 2022; Zhang et al., 2024a). OOD detection is the task of detecting unknown samples during inference to ensure the safety of the in-distribution (ID) classifiers. Along with the evolution of the close-set classifiers, the target tasks for OOD detection have evolved from the detectors for conventional single-modal classifiers to recent CLIP-based methods (Miyai et al., 2024; Hendrycks and Gimpel, 2017; Yu and Aizawa, 2019; Wang et al., 2021; Du et al., 2022; Ming et al., 2022b; Esmaeilpour et al., 2022; Ming et al., 2022a; Yang et al., 2023; Wang et al., 2023a; Miyai et al., 2023a,b). The next crucial challenge is to evolve the problems faced in OOD detection to LMMs in the VQA task. We consider that our UPD is an extension of the concept of OOD detection, where the model should detect and not predict unexpected input data.
+## B Benchmark Construction
+We carefully adapt MMBench (validation) to create our MM-UPD Bench. For simplicity of explanation, we show the mapping table of each index and each ability in MMBench in Table A. MMBench (20231003) is a VQA dataset consisting of 1,164 questions. To create the MM-UPD Bench from MMBench, we conduct the following processes.
+## B.1 Processing for MMBench Adaptation
+First, we performed the following steps for the original MMBench to ensure the quality of our benchmarks.
+</t>
+  </si>
+  <si>
+    <t>Not found in context.</t>
+  </si>
+  <si>
+    <t>Yes – the experiment shows that self‑reflection enables LLMs to judge and evaluate their own answers.</t>
+  </si>
+  <si>
+    <t>Rock climbing.</t>
+  </si>
+  <si>
+    <t>Yes – the curation process requires a detailed justification for any refinement. Each problem that needs adjustment is documented with a reason in the comment field, and disagreements are resolved through discussion and consensus among the annotators.</t>
+  </si>
+  <si>
+    <t>Yes. The context notes that self‑reflection “allows the model to reflect on its own responses” and that LLMs have shown preliminary capabilities for judging and evaluating their own answers.</t>
   </si>
 </sst>
 </file>
@@ -409,10 +630,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -422,49 +643,79 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>10</v>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
the code is as messy as how I feel
</commit_message>
<xml_diff>
--- a/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
+++ b/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>query</t>
   </si>
@@ -289,16 +289,19 @@
     <t>Not found in context.</t>
   </si>
   <si>
-    <t>Yes – the experiment shows that self‑reflection enables LLMs to judge and evaluate their own answers.</t>
+    <t>Yes. The self‑reflection prompt is designed to let the LMM judge its own answer—if it declares “2. False,” the answer is withdrawn, indicating that the model is evaluating its response.</t>
   </si>
   <si>
     <t>Rock climbing.</t>
   </si>
   <si>
-    <t>Yes – the curation process requires a detailed justification for any refinement. Each problem that needs adjustment is documented with a reason in the comment field, and disagreements are resolved through discussion and consensus among the annotators.</t>
-  </si>
-  <si>
-    <t>Yes. The context notes that self‑reflection “allows the model to reflect on its own responses” and that LLMs have shown preliminary capabilities for judging and evaluating their own answers.</t>
+    <t>Yes. The process requires that any refinement is accompanied by a detailed justification recorded as a comment.</t>
+  </si>
+  <si>
+    <t>Yes – the self‑reflection approach is designed to let models judge and evaluate their own answers.</t>
+  </si>
+  <si>
+    <t>Cliff climbing (commonly called rock climbing).</t>
   </si>
 </sst>
 </file>
@@ -715,7 +718,7 @@
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
at least fixed the bug for latest libraries
</commit_message>
<xml_diff>
--- a/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
+++ b/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>query</t>
   </si>
@@ -289,19 +289,16 @@
     <t>Not found in context.</t>
   </si>
   <si>
-    <t>Yes. The self‑reflection prompt is designed to let the LMM judge its own answer—if it declares “2. False,” the answer is withdrawn, indicating that the model is evaluating its response.</t>
+    <t>Yes. The self‑reflection prompt is designed to let the model assess and judge its own answer, and prior work suggests LLMs have preliminary capabilities for this self‑evaluation.</t>
   </si>
   <si>
     <t>Rock climbing.</t>
   </si>
   <si>
-    <t>Yes. The process requires that any refinement is accompanied by a detailed justification recorded as a comment.</t>
-  </si>
-  <si>
-    <t>Yes – the self‑reflection approach is designed to let models judge and evaluate their own answers.</t>
-  </si>
-  <si>
-    <t>Cliff climbing (commonly called rock climbing).</t>
+    <t>Yes. When a problem needs refining, the reason must be recorded in detail as a comment, and if annotators disagree, all four discuss and reach consensus, ensuring thorough justification.</t>
+  </si>
+  <si>
+    <t>Yes. The text states that self‑reflection allows the model to judge and evaluate its own responses (Kadavath et al., 2022; Feng et al., 2024).</t>
   </si>
 </sst>
 </file>
@@ -718,7 +715,7 @@
         <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add answer quality results
</commit_message>
<xml_diff>
--- a/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
+++ b/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
@@ -289,16 +289,16 @@
     <t>Not found in context.</t>
   </si>
   <si>
-    <t>Yes. The self‑reflection prompt is designed to let the model assess and judge its own answer, and prior work suggests LLMs have preliminary capabilities for this self‑evaluation.</t>
+    <t>Yes. The passage explains that self‑reflection “is a method that allows the model to reflect on its own responses” and that LLMs “might have preliminary capabilities for judging and evaluating their own answers.”</t>
   </si>
   <si>
     <t>Rock climbing.</t>
   </si>
   <si>
-    <t>Yes. When a problem needs refining, the reason must be recorded in detail as a comment, and if annotators disagree, all four discuss and reach consensus, ensuring thorough justification.</t>
-  </si>
-  <si>
-    <t>Yes. The text states that self‑reflection allows the model to judge and evaluate its own responses (Kadavath et al., 2022; Feng et al., 2024).</t>
+    <t>Yes – when a problem is refined, the reason is recorded in detail as a comment, and all annotators discuss it to reach consensus.</t>
+  </si>
+  <si>
+    <t>Yes—self‑reflection enables models to judge and evaluate the answers they generate.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
adjusted answer eval logic
</commit_message>
<xml_diff>
--- a/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
+++ b/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
   <si>
     <t>query</t>
   </si>
@@ -22,13 +22,43 @@
     <t>top1_retrieved_chunk_docling</t>
   </si>
   <si>
+    <t>retrieval_score_docling</t>
+  </si>
+  <si>
+    <t>rr_reasoning_docling</t>
+  </si>
+  <si>
+    <t>answer_docling</t>
+  </si>
+  <si>
+    <t>answer_quality_score_docling</t>
+  </si>
+  <si>
+    <t>aq_grounded_docling</t>
+  </si>
+  <si>
+    <t>aq_reasoning_docling</t>
+  </si>
+  <si>
     <t>top1_retrieved_chunk_mineru</t>
   </si>
   <si>
-    <t>answer_docling</t>
+    <t>retrieval_score_mineru</t>
+  </si>
+  <si>
+    <t>rr_reasoning_mineru</t>
   </si>
   <si>
     <t>answer_mineru</t>
+  </si>
+  <si>
+    <t>answer_quality_score_mineru</t>
+  </si>
+  <si>
+    <t>aq_grounded_mineru</t>
+  </si>
+  <si>
+    <t>aq_reasoning_mineru</t>
   </si>
   <si>
     <t>Is detailed justification required when refining problems during the curation process?</t>
@@ -118,6 +148,42 @@
 Table H: Full results for AAD in the base setting. We report Standard accuracy, AAD accuracy, and Dual accuracy.
 | #18   | 0.0 11.4 25.0 2.3 4.5 0.0 0.0 0.0 0.0 0.0 0.0 9.1 9.1 20.5 0.0 2.3 13.6 0.0 31.8 38.6 20.5 43.2                                                                                                                                                              | 0.0 22.7 31.8 4.5 6.8 0.0 0.0 2.3 0.0 0.0 0.0 11.4 11.4 27.3 0.0 2.3 18.2 0.0 34.1 43.2 25.0 45.5                                                                                                                                                                         | 18.2 22.7 50.0 6.8 43.2 6.8 27.3 25.0 34.1 43.2 47.7 27.3 45.5 59.1 27.3 47.7 70.5 47.7 77.3 72.7 68.2 75.0                                                                                                                                        |
 </t>
+  </si>
+  <si>
+    <t>The chunk discusses LMM evaluation methods and experimental details, with no mention of justification or problem refinement in curation.</t>
+  </si>
+  <si>
+    <t>The chunk references a figure titled "Relationship between OC‑Dual accuracy and Dual accuracy," indicating relevance to the query. However, it provides no textual detail about the correlation strength, so it offers only partial information.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly discusses self‑reflection as a method for models to evaluate their own responses, citing studies that show preliminary capabilities for judging answers. It directly addresses the query and provides sufficient detail.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly mentions rock climbing, describing friends using ropes and harnesses on a cliff face, directly answering the query.</t>
+  </si>
+  <si>
+    <t>Not found in context.</t>
+  </si>
+  <si>
+    <t>Yes – the figure shows a strong positive correlation between OC‑Dual accuracy and Dual accuracy.</t>
+  </si>
+  <si>
+    <t>Yes. The self‑reflection prompt asks the model to judge its own answer; if it outputs “2. False” the response is withdrawn, otherwise the original answer is kept.</t>
+  </si>
+  <si>
+    <t>Rock climbing.</t>
+  </si>
+  <si>
+    <t>The answer does not address the user’s question about detailed justification during problem refinement.</t>
+  </si>
+  <si>
+    <t>The answer directly confirms a strong positive correlation, matching the retrieved figure that depicts the relationship. It fully addresses the query and is consistent with the provided context.</t>
+  </si>
+  <si>
+    <t>The answer directly confirms that self‑reflection enables a model to evaluate its own answer, matching the query. The retrieved chunk explicitly describes self‑reflection as a method for models to judge their responses, so the answer is consistent with the context.</t>
+  </si>
+  <si>
+    <t>The answer "Rock climbing" directly answers the query about an activity that uses ropes and harnesses on a cliff face. The retrieved chunk contains a statement describing rock climbing with ropes and harnesses, so the answer is consistent with the context.</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -286,19 +352,34 @@
 </t>
   </si>
   <si>
-    <t>Not found in context.</t>
-  </si>
-  <si>
-    <t>Yes. The passage explains that self‑reflection “is a method that allows the model to reflect on its own responses” and that LLMs “might have preliminary capabilities for judging and evaluating their own answers.”</t>
-  </si>
-  <si>
-    <t>Rock climbing.</t>
-  </si>
-  <si>
-    <t>Yes – when a problem is refined, the reason is recorded in detail as a comment, and all annotators discuss it to reach consensus.</t>
-  </si>
-  <si>
-    <t>Yes—self‑reflection enables models to judge and evaluate the answers they generate.</t>
+    <t>The chunk explicitly describes that when refining problems, annotators record detailed justifications in comments, discuss disagreements, and reach consensus, directly addressing the query about the need for detailed justification during curation.</t>
+  </si>
+  <si>
+    <t>The chunk discusses Dual accuracy but does not mention OC‑Dual accuracy or any correlation between the two metrics, so it only loosely relates to the query.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly states that self‑reflection enables models to judge and evaluate their own answers, directly answering the query.</t>
+  </si>
+  <si>
+    <t>The chunk contains a bibliography of AI research papers and does not mention ropes, harnesses, cliff faces, or any climbing activity. It is completely unrelated to the query.</t>
+  </si>
+  <si>
+    <t>Yes – when a problem is refined during curation, the reason must be recorded in detail as a comment, ensuring a clear justification for the change.</t>
+  </si>
+  <si>
+    <t>Yes – the text explains that self‑reflection lets the model look at its own output, and prior work has shown that LLMs can preliminarily judge and evaluate their answers.</t>
+  </si>
+  <si>
+    <t>The answer directly confirms that detailed justification is required and cites the same practice described in the retrieved chunk, fully addressing the query.</t>
+  </si>
+  <si>
+    <t>The answer does not address the question about the correlation between OC-Dual accuracy and Dual accuracy.</t>
+  </si>
+  <si>
+    <t>The answer directly confirms that self‑reflection enables models to evaluate their own answers, matching the retrieved text that states LLMs can judge and evaluate their responses.</t>
+  </si>
+  <si>
+    <t>The answer correctly identifies rock climbing as the activity that uses ropes and harnesses on a cliff face, fully addressing the user’s question. However, the retrieved chunk is irrelevant (relevancy score 0), so grounding cannot be assessed.</t>
   </si>
 </sst>
 </file>
@@ -630,10 +711,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -649,73 +730,214 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
+        <v>19</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2">
+        <v>3</v>
+      </c>
+      <c r="K2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
         <v>19</v>
       </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" t="s">
+        <v>43</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="s">
+        <v>46</v>
+      </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>29</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
+      </c>
+      <c r="O5" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
10 queries in total
</commit_message>
<xml_diff>
--- a/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
+++ b/experiments_multimodal/pdf_parsing/docling_vs_mineru_qa_comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="96">
   <si>
     <t>query</t>
   </si>
@@ -61,6 +61,9 @@
     <t>aq_reasoning_mineru</t>
   </si>
   <si>
+    <t>What does MM-UPD Bench stand for?</t>
+  </si>
+  <si>
     <t>Is detailed justification required when refining problems during the curation process?</t>
   </si>
   <si>
@@ -71,6 +74,60 @@
   </si>
   <si>
     <t>What activity involves using ropes and harnesses on a cliff face?</t>
+  </si>
+  <si>
+    <t>Why is Dual accuracy considered effective for assessing LMMs' reliability?</t>
+  </si>
+  <si>
+    <t>What is the purpose of Unsolvable Problem Detection (UPD)?</t>
+  </si>
+  <si>
+    <t>Does UPD-specific training affect the performance of general tasks?</t>
+  </si>
+  <si>
+    <t>Do closed-source models offer a better response than open-source models in this evaluation?</t>
+  </si>
+  <si>
+    <t>How does UPD differ from traditional multiple-choice question answering for LMMs?</t>
+  </si>
+  <si>
+    <t>## Unsolvable Problem Detection: Robust Understanding Evaluation for Large Multimodal Models
+Atsuyuki Miyai 1 Jingkang Yang 2 Jingyang Zhang 3 Yifei Ming 4 Qing Yu 1 , 5 Go Irie 6 Yixuan Li 4 Hai Li 3 Ziwei Liu 2 Kiyoharu Aizawa 1 1 The University of Tokyo 2 S-Lab, Nanyang Technological University 3 Duke University 4 University of Wisconsin-Madison 5 LY Corporation 6 Tokyo University of Science
+https://github.com/AtsuMiyai/UPD
+## Abstract
+This paper introduces a novel task to evaluate the robust understanding capability of Large Multimodal Models (LMMs), termed Unsolvable Problem Detection (UPD) . Multiplechoice question answering (MCQA) is widely used to assess the understanding capability of LMMs, but it does not guarantee that LMMs truly comprehend the answer. UPD assesses the LMM's ability to withhold answers when encountering unsolvable problems of MCQA, verifying whether the model truly understands the answer. UPD encompasses three problems: Absent Answer Detection (AAD), Incompatible Answer Set Detection (IASD), and Incompatible Visual Question Detection (IVQD), covering unsolvable cases like answer-lacking or incompatible choices and image-question mismatches. For the evaluation, we introduce the MM-UPD Bench, a benchmark for assessing performance across various ability dimensions. Our experiments reveal that even most LMMs, which demonstrate adequate performance on existing benchmarks, struggle significantly with MM-UPD, underscoring a novel aspect of trustworthiness that current benchmarks have overlooked. A detailed analysis shows that LMMs have different bottlenecks and chain-of-thought and self-reflection improved performance for LMMs with the bottleneck in their LLM capability. We hope our insights will enhance the broader understanding and development of more reliable LMMs.
+## 1 Introduction
+In recent years, following the revolutionary development of Large Language Models (LLMs) (Chen et al., 2024a; Chiang et al., 2023; Touvron et al., 2023; Wei et al., 2023), Large Multimodal Models (LMMs) (Liu et al., 2024c; Wang et al., 2023c; Hurst et al., 2024) have also demonstrated profound capabilities in various applications and sig- nificantly enhance the performance in image reasoning tasks (Antol et al., 2015; Liu et al., 2024b,e; Yue et al., 2024a).
+(c) Incompatible Visual Question Detection (IVQD)
+&lt;!-- image --&gt;
+Figure 1: The Unsolvable Problem Detection (UPD) Challenges . Current Large Multimodal Models (LMMs) like LLaVA-OneVision show adequate performance (blue) on standard problems (MMBench) where an answer is guaranteed. However, they exhibit a notable deficiency (red) refraining from answering unsolvable problems.
+Assessing the understanding capability of LMMs is crucial for advancing fundamental progress. Multiple-Choice Question Answering (MCQA) serves as a fundamental format for understanding evaluation and is widely used in wellestablished benchmarks such as MMBench (Liu et al., 2024e) and MMMU (Yue et al., 2024a). Each MCQA instance consists of a question paired with multiple answer options, requiring models to select the correct one. MCQA enables precise evaluation of LMMs and facilitates solid progress in the field. Consequently, many MCQA-based benchmarks have been proposed recently (Fu et al., 2024; Yue et al., 2024b; Hu et al., 2025).
+Despite the advanced performance of LMMs on the accuracy of MCQA-format benchmarks, concerns remain regarding the reliability of their predictions. While previous works in the field of LLMs have discussed challenges such as maintaining invariance to different orderings of answer choices (Robinson et al., 2023; Wang et al., 2024a; Zheng et al., 2025), overcoming order sensitivity alone is not sufficient to ensure that the model truly understands the correct answer. A more recent study (Wang et al., 2025) investigated LLMs' ability to reject unsolvable problems, such as questions where the correct answer is not present among the given choices. The ability to reject unsolvable problems can serve as a more reliable means of verifying the model's true understanding. However, this study does not focus on LMMs. When extending the evaluation from LLMs to LMMs, the types of unsolvable problems differ. Additionally, there is a lack of benchmarks and systematic evaluation protocols for comprehensively assessing recent LMMs. Consequently, existing works fail to assess the depth of LMMs' robust comprehension.
+To assess the robust comprehension of LMMs, we propose Unsolvable Problem Detection (UPD), which examines the LMM's ability to withhold answers when faced with unsolvable problems. UPD encompasses three distinct settings: Absent Answer Detection (AAD), Incompatible Answer Set Detection (IASD), and Incompatible Visual Question Detection (IVQD). Fig. 1 shows the illustration of each setting. AAD evaluates whether the model declines to provide an answer when the correct answer is absent. IASD examines whether the model rejects a question when the given answer set is entirely incompatible. IVQD investigates the model's ability to reject a question when there is no relevance between the image and the text question. A model that effectively rejects unsolvable problems while accurately solving standard solvable problems can be regarded as truly understanding them. On the other hand, a model that incorrectly selects an answer for unsolvable problems cannot be considered to have a true understanding of them.
+For the evaluation, we introduce MM-UPD Bench , a carefully designed benchmark for evalu- ating UPD capability across various ability dimensions. MM-UPD employs a rigorous three-step construction process that builds upon MMBench (Liu et al., 2024e): (1) filtering out questions that can be answered by text-only language models, (2) applying the carefully designed approach for creating UPD questions, (3) finally, manually removing ambiguous samples. Built on the foundation of MMBench, our benchmarks allow us to highlight the difficulty of MM-UPD by comparing it to the self-established MMBench, and also serves as a fine-grained diagnostic tool, offering detailed insights into each LMM's weaknesses in a broad range of MMBench's abilities.
+Our experimental results demonstrate the difficulty of MM-UPD across various state-of-the-art LMMs. The most important finding is that there is little correlation between the performance on the existing MMBench and MM-UPD Bench. This indicates that the community's efforts to improve performance on existing benchmarks do not directly contribute to enhancing model reliability. In particular, we found that the gap between open-source and closed-source models is large, while opensource LMMs outperform closed-source LMMs on MMBench. Furthermore, our fine-grained ability analysis revealed that even closed-source models such as GPT-4o (Hurst et al., 2024) exhibit weaknesses in specific abilities.
+Finally, we revealed that whether the bottleneck lies in the LLM's refusal capability or its visual understanding depends on the specific LMM. For LMMs where the bottleneck is in the LLM's refusal capability, we observed performance improvements with LLM-driven approaches such as chain-of-thought (Kojima et al., 2022) and selfreflection (Kadavath et al., 2022).
+Our contributions are summarized as follows:
+- Definition of Unsolvable Problem Detection : We propose a novel challenge called Unsolvable Problem Detection, which evaluates the LMM's robust understanding in three problem settings: AAD, IASD, and IVQD.
+- Construction of MM-UPD Bench : We rigorously construct the MM-UPD Bench and provide a fine-grained diagnostic tool for broader abilities.
+- Benchmarking with Recent LMMs : We evaluate state-of-the-art LMMs on the UPD
+problem and show that our benchmarks represent a new and meaningful dimension of the performances of LMMs.
+## 2 Related Work
+Vulnerability of MCQA Evaluation. The vulnerability of MCQA has mainly been researched in the field of LLM. Previous work has aimed to mitigate bias in answer options and enhance LLMs' consistency across different option orders (Robinson et al., 2023; Wang et al., 2024a; Zheng et al., 2025). As a more recent work, Wang et al. (2025) tested LLM's ability to refuse unsolvable problems. They found that LLMs may perform MCQA by selecting the least incorrect option rather than distinctly correct. However, it only deals with AAD, and when applied to LMMs, the types of unsolvable problems are limited. Additionally, we consider that handling unsolvable problems requires rigorous evaluation based on ability-specific assessments, while they have not clearly identified the performance differences across abilities.
+Unsolvable Problems. Unsolvable questions have been studied in NLP (Rajpurkar et al., 2018; Choi et al., 2018; Reddy et al., 2019; Sulem et al., 2022) and in VQA before the rise of LMMs (Gurari et al., 2018; Bhattacharya et al., 2019; Davis, 2020; Whitehead et al., 2022). Early VQA studies focused on task-specific models, making their benchmarks misaligned with modern LMMs due to task simplicity or differing evaluation protocols. While recent works have explored unsolvable questions in LMMs (Guo et al., 2024; Akter et al., 2024; Cao et al., 2024), they do not assess the robustness of LMMs for common MCQA.
+Answer Refusal. In the task of refusing to provide an answer, there are studies in the field of LLMs that focus on abstaining due to a lack of knowledge (Kadavath et al., 2022; Feng et al., 2024). The main difference between their work and ours is that while they focus on knowledge gaps, we focus on the flaws or incompleteness of the problem itself, which leads to a different problem formulation.
+## 3 Problem Definition
+In this section, we introduce the concept of Unsolvable Problem Detection (UPD), a task designed to evaluate models' capacity to not blindly offer incorrect answers when presented with unsolvable problems. We consider various discrepancies among the provided image, question, and answer options.
+Then, we categorize UPD into three distinct problem types: Absent Answer Detection (AAD), Incompatible Answer Set Detection (IASD), and Incompatible Visual Question Detection (IVQD). Here, AAD has been proposed as an unsolvable type for LLMs in existing work (Wang et al., 2025), but it has not been examined with LMMs. Additionally, by incorporating IASD and IVQD, we can cover a broader scope of unsolvable types, enabling a more precise diagnosis of model weaknesses. The details of each setting are as follows:
+1. Absent Answer Detection (AAD) : AAD tests the model's capability to recognize when the correct answer is absent from the provided choices. It challenges the model to not only analyze the content of questions and images but also identify when it cannot select a correct response due to the absence of an appropriate option.
+2. Incompatible Answer Set Detection (IASD) : IASD tests the model's ability to identify situations where the set of answer choices is incompatible with the context. Differing from AAD, in which the answer set is related to the question or the image, IASD deals with answer sets that are entirely irrelevant, challenging the model to withhold a response due to the lack of reasonable options. By giving a completely unrelated answer set, IASD evaluates the inherent capacity of LMMs to withhold answering, which is not affected by the granularity of the given choices.
+3. Incompatible Visual Question Detection (IVQD) : IVQD evaluates the LMMs' capability to discern when a question and image are irrelevant or inappropriate. This setting tests the model's understanding of the alignment between visual content and textual questions, aiming to spot instances where image-question pairs are incompatible.
+## 4 Benchmarks and Evaluations
+## 4.1 Construction of MM-UPD Bench
+We create MM-UPD Bench based on MMBench (dev, 20231003) (Liu et al., 2024e). MMBench (Liu et al., 2024e) is a systematically designed benchmark for evaluating various abilities of LMMs. Utilizing MMBench allows us to assess the reliability of LMMs for general VQA questions and also enables fine-grained, ability-wise evaluation ( e.g., , 'Coarse Perception: Image Scene' and 'Logic Reasoning: Future Prediction').
+To create MM-UPD Bench, we first filter imageagnostic questions from MMBench.
+Figure 2: Examples of standard and UPD questions in each scenario. We evaluate all 4 four scenarios (Standard, AAD, IASD, and IVQD) as follows: the base setting, where no UPD-specific options/instructions are provided; the Option setting, which includes an option like 'None of the above"; and the Instruction setting, where explicit guidance such as 'Answer F. None of the above" is given. We calculate the Dual accuracy with the prediction of each Standard-UPD question pair ( e.g., Standard-base and AAD-base).
+&lt;!-- image --&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -150,40 +207,149 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">
+F3: UPD Score is Significantly Lower than Standard in Base and Solution Varies by LMMs. Fig. 3 shows the Standard (blue) and UPD (red) accuracy. The performance was compared, with each row showing the results for AAD, IASD, and IVQD, and each column showing the results for Base, Option, and Instruction. Models (i)-(v) in the figure denotes open-source models and Model (vi)-(viii) denotes closed-source models. First, for the Base settings, open-source LMMs indeed exhibit lower UPD accuracy compared to Standard accuracy. Even for the Option setting, open-source LMMs still tend to perform worse on UPD than on Standard. When additional instruction is added, some models finally show a reversal in UPD and Standard performance. However, for (i) LLaVAOV-7B and (iii) InternVL2-8B, the UPD accuracy decreases compared to the Option setting. Therefore, effective prompting strategies to refrain from providing answers vary by LMMs.
+F4: Performance of AAD, IASD, and IVQD
+Table 3: Overall Dual accuracy with chain of thought prompting and self-reflection. The values in () represent Standard accuracy and UPD accuracy, respectively.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+## D.1 Setup
+Dataset. For the dataset, we use a subset of an open-knowledge VQA dataset, AOKVQA (Schwenk et al., 2022). It is a singlechoice type VQA dataset that has been used for training InstructBLIP (Dai et al., 2023) and LLaV A1.5 (Liu et al., 2024c). The samples in A-OKVQA do not overlap with our benchmarks.
+To address all three types of problems, the ratio of the tuning data for each task is important. Therefore, we examine the difficulty and heterogeneity of each task and then seek the optimal amount and proportion of each type of question. We first create 4 kinds of datasets for standard questions, AAD questions, IASD questions, and IVQD questions, respectively. For each dataset, we include the questions for the base setting and the questions with additional options. For AAD/IASD/IVQD datasets, we set 'I cannot answer.' as the answer for the base-setting questions and set the UPD-specific options such as 'None of the above' to the answer for the option-setting questions. Also, to make it robust for the number of options, we create the questions with 2-4 options by augmentations.
+Model and Tuning Method. The experiments were conducted based on LLaVA-NeXT-13B/34B
+due to its ease of implementation and its powerful performance. We adopt LoRA tuning (Hu et al., 2022) by considering the effectiveness and low memory usage.
+## D.2 Analysis
+In this section, we aim to explore the optimal tuning recipe. First, we investigate the difficulty and heterogeneity of the AAD, IASD, and IVQD tasks. Then, by conducting experiments with varying proportions of each task and adjusting the amount of data, we identify the best tuning recipe.
+Difficulty and Heterogeneity of Each Task. To create a dataset that addresses all UPD problems, it is crucial to examine the difficulty and heterogeneity of each task. To this end, we compare the performances when we use only one UPD dataset from all three kinds of UPD datasets, which indicates the difficulty or similarity of each task. In Table G, we show the result. From this result, we find that, for AAD and IVQD, we need to include their own training data, while both IVQD and AAD data are sufficient to solve IASD questions. This is because IASD can be considered a simpler version of the AAD question since the answer-set does not include the correct answer, and it is also related to IVQD since the answer-set is not related to the given image. Hence, to reduce the complexity, we can create the tuning dataset from AAD and IVQD data.
+(a) LLaVA-NeXT-13B
+|      |   Orig before |   Orig after |   Base |   Opt |   Inst |   Inst Tuning |
+|------|---------------|--------------|--------|-------|--------|---------------|
+| AAD  |          76.7 |         68.9 |   18.3 |  18.2 |   38.8 |          47.6 |
+| IASD |          73.2 |         65.4 |   31.4 |  29.8 |   57.8 |          60.0 |
+| IVQD |          71.3 |         67.4 |   29.8 |  37.9 |   54.2 |          59.6 |
+(b) LLaVA-NeXT-34B
+Table E: Overall Dual accuracy with UPD instruction tuning.
+|      |   Orig before |   Orig after |   Base |   Opt |   Inst |   Inst Tuning |
+|------|---------------|--------------|--------|-------|--------|---------------|
+| AAD  |          84.3 |         78.6 |   53.2 |  29.9 |   55.2 |          63.8 |
+| IASD |          80.2 |         74.8 |   56.7 |  22.6 |   61.9 |          73.3 |
+| IVQD |          80.9 |         74.7 |   53.4 |  50.6 |   72.5 |          70.2 |
+Ablation on Ratio of Each UPD Task. In Fig. B, we illustrate the relationship between the ratio of Standard, AAD, and IVQD instruction tuning data and the performance of each UPD, Standard, and Dual accuracy. We set the ratio of Standard: AAD: IVQD to 3.3:3.3:3.3, 6:2:2, 7:2:1, 1:0:0. From this result, increasing the ratio of UPD tuning data, the UPD performance improved much while the standard accuracy degrades. Conversely, increasing the proportion of Standard data degrades the UPD performance. We can see that the ratio of 6:2:2 is an effective ratio for all the settings.
+Ablation on Data Size. In Fig. C, we illustrate the relationship between the tuning data size and the performance of each UPD, Standard, and Dual accuracy. In this experiment, we set the ratio of Standard, AAD, and IVQD is 0.6, 0.2, and 0.2. From this result, 10,000 samples are enough to tune for our LoRA-based instruction tuning.
+From these experiments, we find that the most effective approach is to include 20% AAD and 20% IVQD questions each, and 10,000 samples are sufficient for tuning.
+## D.3 Result
+Table E demonstrates that instruction tuning is effective for UPD, showing the performance efficacy and limitations with UPD-specific training. However, UPD-specific training may degrade the performance of other general tasks. Therefore, if the user intends to use LMMs for broader, more general purposes rather than just for UPD tasks, instruction tuning may not be a good approach. It is a future challenge to propose a method that improves UPD performance while maintaining performance on general tasks.
+## E Evaluation
+## E.1 Further Discussion of Evaluation Metrics
+We consider the Original Conditional Dual accuracy (OC-Dual) score, a metric that takes into account the Original Standard Accuracy for each LMM. Dual Accuracy is an evaluation metric that equally assesses Standard accuracy and UPD accuracy. This metric inherits the widely supported concept of a reliable model that answers when it should and refuses when it should not (Amodei et al., 2016; Hendrycks et al., 2021; Yang et al., 2024b). However, it also takes into account differences in the original capability for Standard problems. Therefore, we consider the OC-Dual score as a score that does not depend on the original capability. The OC-Dual score is defined as follows: OC-Dual = (Success in all Original Standard, Standard, UPD settings) / (Success in Original Standard).
+We plotted the relationship between OC-Dual accuracy and Dual accuracy in Fig A. To quantify the relationship between these scores, we calculated the correlation coefficient ( r ) and Spearman's rank correlation coefficient ( ρ ). The analysis revealed a very strong correlation between the two metrics. This is attributed to the fact that the Original Standard performance of current LMMs shows little variation within the MM-UPD Bench. Given that OC-Dual accuracy does not guarantee practical usability, the Dual accuracy for MM-UPD is the most effective to precisely assess the reliability of state-of-the-art LMMs without compromising real-world applicability.
+## E.2 Automatic Evaluation Strategy
+We adopt Circular Evaluation and GPT-involved Choice Extraction in MMBench (Liu et al., 2024e) as an evaluation strategy. In Circular Evaluation, a problem is tested multiple times with circularly shifted choices, and the LMM needs to succeed in all testing passes. GPT-involved Choice Extraction first performs the matching algorithm and then uses GPT for those that do not match.
+However, since the existing MMBench evalua- tions are optimized for standard questions, directly using them would assign standard options to refusal responses. Therefore, we made the following modifications for the UPD challenge.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+F1: Different Performance Trends of MMBench and MM-UPD Bench. Table 1 shows that the performance trends of MMBench (Orig) and MM-UPD (Base/Opt/Inst) are completely different. For instance, although LLaVA-OV-7B (Li et al., 2024a), CogVLM2 (Hong et al., 2024), and XgenMM (Xue et al., 2024) exhibit very high performance ( &amp;gt; 80%) in all Original Standard, their performances in the UPD Base setting drop to less than 6% in all Base settings. To investigate the correlation more rigorously, we calculate the correlation coefficients between the Original Standard and Dual accuracy/UPD accuracy in Table 2. We found that the correlation coefficient between UPD accuracy and the Original Standard is quite low (Max: 39.1, Min: 6.5). Dual accuracies still do not indicate a strong correlation. This suggests that our benchmark is capable of accurately capturing an important aspect of trustworthiness that has not been measured by previous benchmarks.
+F2: Large Gap between Open-source LMMs and Closed-source LMMs. As shown in Table 1, there is a significant performance gap between open-source LMMs and closed-source LMMs. One of the reasons for this performance gap is the training difference: Closed-source models are trained for refusal considering real-world user applications according to their system cards (Hurst et al., 2024; OpenAI, 2023). On the other hand, open-source models usually compete for performance with limited publicly available benchmarks. However, among open-source LMMs, models with large LLMs such as LLaVA-NeXT-34B and InternVL2-40B demonstrate performance comparable to closed-source models. Compared to smaller models trained on the same VQA data, such as LLaVA-NeXT-13B and InternVL2-2B/8B, there is a significant performance improvement, suggesting that the performance of the base LLM also plays a crucial role. However, a detailed check of each output reveals that a quality gap still exists between these powerful open-source LMMs and closed-source LMMs (refer to Appendix F.2).
+Next, we provide detailed findings below to support the rationale behind the above findings.
+</t>
+  </si>
+  <si>
+    <t>The chunk mentions MM‑UPD Bench as a benchmark for unsolvable problem detection, but it does not explain what the acronym MM‑UPD Bench expands to, so it only loosely relates to the query.</t>
+  </si>
+  <si>
     <t>The chunk discusses LMM evaluation methods and experimental details, with no mention of justification or problem refinement in curation.</t>
   </si>
   <si>
-    <t>The chunk references a figure titled "Relationship between OC‑Dual accuracy and Dual accuracy," indicating relevance to the query. However, it provides no textual detail about the correlation strength, so it offers only partial information.</t>
-  </si>
-  <si>
-    <t>The chunk explicitly discusses self‑reflection as a method for models to evaluate their own responses, citing studies that show preliminary capabilities for judging answers. It directly addresses the query and provides sufficient detail.</t>
-  </si>
-  <si>
-    <t>The chunk explicitly mentions rock climbing, describing friends using ropes and harnesses on a cliff face, directly answering the query.</t>
+    <t>The chunk references a figure titled "Relationship between OC‑Dual accuracy and Dual accuracy," indicating relevance to the query. However, it provides no textual detail on the correlation strength, so it offers only partial information.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly discusses self‑reflection as a method for models to evaluate their own responses, citing studies that show preliminary capabilities for judging and evaluating answers. It directly addresses the query and provides sufficient detail to answer it.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly mentions "rock climbing" as an activity that uses ropes and harnesses on a cliff face, directly answering the query.</t>
+  </si>
+  <si>
+    <t>The chunk mentions Dual accuracy and compares UPD vs Standard accuracy, indicating its use in evaluating LMMs, but it does not explain why Dual accuracy is considered effective for assessing reliability.</t>
+  </si>
+  <si>
+    <t>The chunk explains UPD’s goal of testing LMMs’ ability to refuse unsolvable MCQA problems, detailing its purpose and evaluation framework.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly discusses UPD‑specific training and notes that it can degrade performance on general tasks, directly answering the query.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly states a significant performance gap favoring closed‑source LMMs over open‑source ones in the evaluation, directly answering the query.</t>
+  </si>
+  <si>
+    <t>The chunk explains UPD as a task that tests LMMs’ ability to refuse unsolvable MCQA problems, contrasts it with standard MCQA, and details the three unsolvable problem types, directly answering how UPD differs from traditional MCQA.</t>
+  </si>
+  <si>
+    <t>**MM‑UPD Bench** stands for the *Multimodal Unsolvable Problem Detection Benchmark*.</t>
   </si>
   <si>
     <t>Not found in context.</t>
   </si>
   <si>
-    <t>Yes – the figure shows a strong positive correlation between OC‑Dual accuracy and Dual accuracy.</t>
-  </si>
-  <si>
-    <t>Yes. The self‑reflection prompt asks the model to judge its own answer; if it outputs “2. False” the response is withdrawn, otherwise the original answer is kept.</t>
+    <t>Yes. The experiments show that self‑reflection lets the model judge and evaluate its own answer, and it can withdraw a response if it judges it to be false.</t>
   </si>
   <si>
     <t>Rock climbing.</t>
   </si>
   <si>
+    <t>Unsolvable Problem Detection (UPD) is designed to evaluate a Large Multimodal Model’s robust understanding by testing whether the model can **recognize unsolvable questions and refuse to answer**. It covers three settings—Absent Answer Detection, Incompatible Answer Set Detection, and Incompatible Visual Question Detection—and measures a model’s ability to withhold responses when the correct answer is missing, irrelevant, or the image‑question pair is mismatched.</t>
+  </si>
+  <si>
+    <t>Yes. The results show that while UPD‑specific instruction tuning boosts UPD performance, it can hurt performance on other general tasks. Consequently, if a model is intended for broader, general use, UPD‑specific training may not be advisable.</t>
+  </si>
+  <si>
+    <t>Yes. According to the context, closed‑source LMMs consistently outperform open‑source ones in this evaluation.</t>
+  </si>
+  <si>
+    <t>UPD is a *robust‑understanding* variant of MCQA that explicitly tests the model’s ability to **abstain** when the question is unsolvable.  
+Unlike standard MCQA, where every item has a correct answer and the model is expected to pick one of the given options, UPD introduces three kinds of “unsolvable” problems:
+1. **Absent Answer Detection (AAD)** – the correct answer is missing from the choice set.  
+2. **Incompatible Answer Set Detection (IASD)** – the entire answer set is irrelevant to the question.  
+3. **Incompatible Visual Question Detection (IVQD)** – the image and the textual question do not match.
+A model that truly understands the task must refuse to answer (or answer “none of the above”) for these cases, rather than forcing a choice or guessing the least‑wrong option. Thus UPD differs from traditional MCQA by measuring a model’s refusal/abstention capability and robustness to poorly‑formed or mismatched inputs.</t>
+  </si>
+  <si>
+    <t>The answer correctly expands MM‑UPD Bench as "Multimodal Unsolvable Problem Detection Benchmark," fully addressing the user’s question. The retrieved chunk does not provide the expansion, so grounding cannot be assessed.</t>
+  </si>
+  <si>
     <t>The answer does not address the user’s question about detailed justification during problem refinement.</t>
   </si>
   <si>
-    <t>The answer directly confirms a strong positive correlation, matching the retrieved figure that depicts the relationship. It fully addresses the query and is consistent with the provided context.</t>
-  </si>
-  <si>
-    <t>The answer directly confirms that self‑reflection enables a model to evaluate its own answer, matching the query. The retrieved chunk explicitly describes self‑reflection as a method for models to judge their responses, so the answer is consistent with the context.</t>
-  </si>
-  <si>
-    <t>The answer "Rock climbing" directly answers the query about an activity that uses ropes and harnesses on a cliff face. The retrieved chunk contains a statement describing rock climbing with ropes and harnesses, so the answer is consistent with the context.</t>
+    <t>The answer does not address the question about the correlation between OC‑Dual accuracy and Dual accuracy, so it scores 0. Since the retrieved chunk is relevant (score 2), we evaluate consistency; the answer provides no information and is therefore not consistent with the context.</t>
+  </si>
+  <si>
+    <t>The answer directly confirms that self‑reflection enables models to judge and evaluate their own answers, matching the retrieved chunk that states LLMs can reflect on responses and assess correctness. It fully addresses the query and is consistent with the source.</t>
+  </si>
+  <si>
+    <t>The answer "Rock climbing" directly answers the question about an activity that uses ropes and harnesses on a cliff face. The retrieved chunk contains a statement describing rock climbing with ropes and harnesses, so the answer is consistent with the context.</t>
+  </si>
+  <si>
+    <t>The answer "Not found in context." does not address the question about why Dual accuracy is effective for assessing LMM reliability, and it provides no information from the retrieved chunk.</t>
+  </si>
+  <si>
+    <t>The answer clearly states that UPD evaluates a model’s robust understanding by testing its ability to recognize unsolvable questions and refuse to answer, and it lists the three settings (AAD, IASD, IVQD). This matches the retrieved chunk’s description, so it fully addresses the query and is consistent with the context.</t>
+  </si>
+  <si>
+    <t>The answer directly states that UPD‑specific training improves UPD performance but can hurt general tasks, matching the query. The retrieved chunk confirms this claim, so the answer is fully correct and grounded.</t>
+  </si>
+  <si>
+    <t>The answer directly states that closed‑source models outperform open‑source ones, matching the retrieved chunk’s claim of a significant performance gap. It fully addresses the user’s question and is consistent with the evidence.</t>
+  </si>
+  <si>
+    <t>The answer fully explains that UPD extends traditional MCQA by adding unsolvable problem types (AAD, IASD, IVQD) and requiring models to abstain rather than guess, directly addressing the query. It aligns with the retrieved paper, which defines UPD, its three settings, and contrasts it with standard MCQA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+&lt;table&gt;&lt;tr&gt;&lt;td rowspan=1 colspan=1&gt;#8&lt;/td&gt;&lt;td rowspan=1 colspan=1&gt;#9&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;#10&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;#11&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;#12&lt;/td&gt;&lt;td rowspan=1 colspan=1&gt;#13&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td rowspan=1 colspan=1&gt;PhysicalRelation&lt;/td&gt;&lt;td rowspan=1 colspan=1&gt;SocialRelation&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;IdentityReasoning&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;FunctionReasoning&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;PhysicalPropertyReasoning&lt;/td&gt;&lt;td rowspan=1 colspan=1&gt;StructuralizedImage-textUnderstanding&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td rowspan=3 colspan=9&gt;#14      #15     #16     #17    #18Future                                   ImagePrediction                                  Style&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td rowspan=1 colspan=1&gt;#15&lt;/td&gt;&lt;td rowspan=1 colspan=1&gt;#16&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;#17&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td rowspan=1 colspan=1&gt;Image&lt;/td&gt;&lt;td rowspan=1 colspan=1&gt;Emage n&lt;/td&gt;&lt;td rowspan=1 colspan=2&gt;Iane&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
+Table A: Mapping table of indices and abilities in MM-UPD Bench</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -352,34 +518,204 @@
 </t>
   </si>
   <si>
+    <t># Unsolvable Problem Detection: Robust Understanding Evaluation for Large Multimodal Models
+Atsuyuki Miyai&lt;sup&gt;1&lt;/sup&gt; Jingkang Yang&lt;sup&gt;2&lt;/sup&gt; Jingyang Zhang&lt;sup&gt;3&lt;/sup&gt; Yifei Ming&lt;sup&gt;4&lt;/sup&gt; Qing Yu&lt;sup&gt;1,5&lt;/sup&gt; Go Irie&lt;sup&gt;6&lt;/sup&gt; Yixuan Li&lt;sup&gt;4&lt;/sup&gt; Hai Li&lt;sup&gt;3&lt;/sup&gt; Ziwei Liu&lt;sup&gt;2&lt;/sup&gt; Kiyoharu Aizawa&lt;sup&gt;1&lt;/sup&gt; &lt;sup&gt;1&lt;/sup&gt;The University of Tokyo &lt;sup&gt;2&lt;/sup&gt;S-Lab, Nanyang Technological University &lt;sup&gt;3&lt;/sup&gt;Duke University &lt;sup&gt;4&lt;/sup&gt;University of Wisconsin-Madison &lt;sup&gt;5&lt;/sup&gt;LY Corporation &lt;sup&gt;6&lt;/sup&gt;Tokyo University of Science
+https://github.com/AtsuMiyai/UPD
+## Abstract
+This paper introduces a novel task to evaluate the robust understanding capability of Large Multimodal Models (LMMs), termed Unsolvable Problem Detection (UPD). Multiplechoice question answering (MCQA) is widely used to assess the understanding capability of LMMs, but it does not guarantee that LMMs truly comprehend the answer. UPD assesses the LMM’s ability to withhold answers when encountering unsolvable problems of MCQA, verifying whether the model truly understands the answer. UPD encompasses three problems: Absent Answer Detection (AAD), Incompatible Answer Set Detection (IASD), and Incompatible Visual Question Detection (IVQD), covering unsolvable cases like answer-lacking or incompatible choices and image-question mismatches. For the evaluation, we introduce the MM-UPD Bench, a benchmark for assessing performance across various ability dimensions. Our experiments reveal that even most LMMs, which demonstrate adequate performance on existing benchmarks, struggle significantly with MM-UPD, underscoring a novel aspect of trustworthiness that current benchmarks have overlooked. A detailed analysis shows that LMMs have different bottlenecks and chain-of-thought and self-reflection im proved performance for LMMs with the bot tleneck in their LLM capability. We hope our insights will enhance the broader understanding and development of more reliable LMMs.
+## 1 Introduction
+In recent years, following the revolutionary development of Large Language Models (LLMs) (Chen et al., 2024a; Chiang et al., 2023; Touvron et al., 2023; Wei et al., 2023), Large Multimodal Models (LMMs) (Liu et al., 2024c; Wang et al., 2023c; Hurst et al., 2024) have also demonstrated profound capabilities in various applications and significantly enhance the performance in image reasoning tasks (Antol et al., 2015; Liu et al., 2024b,e; Yue et al., 2024a).
+![](images/f974a47f88df69e2ec1cb1a3c353029b9081220f2a52a41fb698148e4b5fe901.jpg)  
+(a) Absent Answer Detection (AAD)
+![](images/bb6e79644ac527e3cc0232aba6ebf2a653fc581af4a145321c4a11a082edfd6d.jpg)  
+(b) Incompatible Answer Set Detection (IASD)
+![](images/c908a811ce9eca15b45381c51b72255e4dbf193861e4f6be5b3ca77fd1d07714.jpg)  
+(c) Incompatible Visual Question Detection (IVQD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Table D: Performance comparison on MMMU-AAD. We report overall Dual accuracy. The values in () represent Standard accuracy and UPD accuracy, respectively. ∗: The reason GPT-4o’s Original Standard performance is lower than its Base Standard is that GPT-4o generates extensive long reasoning for challenging datasets like MMMU, solving problems with a chain-of-thought process. However, this arises from GPT-4o’s proprietary tuning strategy and this is unrelated to UPD. Therefore, we omit it from our discussion here.
+## D.1 Setup
+Dataset. For the dataset, we use a subset of an open-knowledge VQA dataset, A-OKVQA (Schwenk et al., 2022). It is a singlechoice type VQA dataset that has been used for training InstructBLIP (Dai et al., 2023) and LLaVA-1.5 (Liu et al., 2024c). The samples in A-OKVQA do not overlap with our benchmarks.
+To address all three types of problems, the ratio of the tuning data for each task is important. Therefore, we examine the difficulty and heterogeneity of each task and then seek the optimal amount and proportion of each type of question. We first create 4 kinds of datasets for standard questions, AAD questions, IASD questions, and IVQD questions, respectively. For each dataset, we include the questions for the base setting and the questions with additional options. For AAD/IASD/IVQD datasets, we set “I cannot answer.” as the answer for the base-setting questions and set the UPD-specific options such as “None of the above” to the answer for the option-setting questions. Also, to make it robust for the number of options, we create the questions with 2-4 options by augmentations.
+Model and Tuning Method. The experiments were conducted based on LLaVA-NeXT-13B/34B due to its ease of implementation and its powerful performance. We adopt LoRA tuning (Hu et al., 2022) by considering the effectiveness and low memory usage.
+## D.2 Analysis
+In this section, we aim to explore the optimal tuning recipe. First, we investigate the difficulty and heterogeneity of the AAD, IASD, and IVQD tasks. Then, by conducting experiments with varying proportions of each task and adjusting the amount of data, we identify the best tuning recipe.
+Difficulty and Heterogeneity of Each Task. To create a dataset that addresses all UPD problems, it is crucial to examine the difficulty and heterogeneity of each task. To this end, we compare the performances when we use only one UPD dataset from all three kinds of UPD datasets, which indicates the difficulty or similarity of each task. In Table G, we show the result. From this result, we find that, for AAD and IVQD, we need to include their own training data, while both IVQD and AAD data are sufficient to solve IASD questions. This is because IASD can be considered a simpler version of the AAD question since the answer-set does not include the correct answer, and it is also related to IVQD since the answer-set is not related to the given image. Hence, to reduce the complexity, we can create the tuning dataset from AAD and IVQD data.
+(a) LLaVA-NeXT-13B
+&lt;table&gt;&lt;tr&gt;&lt;td&gt;&lt;/td&gt;&lt;td&gt;Orig before&lt;/td&gt;&lt;td&gt;Orig after&lt;/td&gt;&lt;td&gt;Base Opt Inst&lt;/td&gt;&lt;td&gt;Inst Tuning&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;AAD IASD IVQD&lt;/td&gt;&lt;td&gt;76.7 73.2&lt;/td&gt;&lt;td&gt;68.9 65.4&lt;/td&gt;&lt;td&gt;18.3 18.2 38.8 31.4 29.8 57.8&lt;/td&gt;&lt;td&gt;47.6 60.0&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
+(b) LLaVA-NeXT-34B
+&lt;table&gt;&lt;tr&gt;&lt;td&gt;&lt;/td&gt;&lt;td&gt;Orig before&lt;/td&gt;&lt;td&gt;Orig after&lt;/td&gt;&lt;td&gt;Base Opt Inst&lt;/td&gt;&lt;td&gt;Inst Tuning&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;AAD&lt;/td&gt;&lt;td&gt;84.3&lt;/td&gt;&lt;td&gt;78.6&lt;/td&gt;&lt;td&gt;53.2 29.9 55.2&lt;/td&gt;&lt;td&gt;63.8&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;IASD&lt;/td&gt;&lt;td&gt;80.2&lt;/td&gt;&lt;td&gt;74.8&lt;/td&gt;&lt;td&gt;56.7 22.6 61.9&lt;/td&gt;&lt;td&gt;73.3&lt;/td&gt;&lt;/tr&gt;&lt;tr&gt;&lt;td&gt;IVQD&lt;/td&gt;&lt;td&gt;80.9&lt;/td&gt;&lt;td&gt;74.7&lt;/td&gt;&lt;td&gt;53.4 50.6 72.5&lt;/td&gt;&lt;td&gt;70.2&lt;/td&gt;&lt;/tr&gt;&lt;/table&gt;
+Table E: Overall Dual accuracy with UPD instruction tuning.
+Ablation on Ratio of Each UPD Task. In Fig. B, we illustrate the relationship between the ratio of Standard, AAD, and IVQD instruction tuning data and the performance of each UPD, Standard, and Dual accuracy. We set the ratio of Standard: AAD: IVQD to 3.3:3.3:3.3, 6:2:2, 7:2:1, 1:0:0. From this result, increasing the ratio of UPD tuning data, the UPD performance improved much while the standard accuracy degrades. Conversely, increasing the proportion of Standard data degrades the UPD performance. We can see that the ratio of 6:2:2 is an effective ratio for all the settings.
+Ablation on Data Size. In Fig. C, we illustrate the relationship between the tuning data size and the performance of each UPD, Standard, and Dual accuracy. In this experiment, we set the ratio of Standard, AAD, and IVQD is 0.6, 0.2, and 0.2. From this result, 10,000 samples are enough to tune for our LoRA-based instruction tuning.
+From these experiments, we find that the most effective approach is to include 20% AAD and 20% IVQD questions each, and 10,000 samples are sufficient for tuning.
+## D.3 Result
+Table E demonstrates that instruction tuning is effective for UPD, showing the performance efficacy and limitations with UPD-specific training. However, UPD-specific training may degrade the performance of other general tasks. Therefore, if the user intends to use LMMs for broader, more general purposes rather than just for UPD tasks, instruction tuning may not be a good approach. It is a future challenge to propose a method that improves UPD performance while maintaining performance on general tasks.
+## E Evaluation
+## E.1 Further Discussion of Evaluation Metrics
+We consider the Original Conditional Dual accuracy (OC-Dual) score, a metric that takes into account the Original Standard Accuracy for each LMM. Dual Accuracy is an evaluation metric that equally assesses Standard accuracy and UPD accuracy. This metric inherits the widely supported concept of a reliable model that answers when it should and refuses when it should not (Amodei et al., 2016; Hendrycks et al., 2021; Yang et al., 2024b). However, it also takes into account differences in the original capability for Standard problems. Therefore, we consider the OC-Dual score as a score that does not depend on the original capability. The OC-Dual score is defined as follows: OC-Dual = (Success in all Original Standard, Standard, UPD settings) / (Success in Original Standard).
+We plotted the relationship between OC-Dual accuracy and Dual accuracy in Fig A. To quantify the relationship between these scores, we calculated the correlation coefficient (r) and Spearman’s rank correlation coefficient (ρ). The analysis revealed a very strong correlation between the two metrics. This is attributed to the fact that the Original Standard performance of current LMMs shows little variation within the MM-UPD Bench. Given that OC-Dual accuracy does not guarantee practical usability, the Dual accuracy for MM-UPD is the most effective to precisely assess the reliability of state-of-the-art LMMs without compromising real-world applicability.
+## E.2 Automatic Evaluation Strategy
+We adopt Circular Evaluation and GPT-involved Choice Extraction in MMBench (Liu et al., 2024e) as an evaluation strategy. In Circular Evaluation, a problem is tested multiple times with circularly shifted choices, and the LMM needs to succeed in all testing passes. GPT-involved Choice Extraction first performs the matching algorithm and then uses GPT for those that do not match.
+However, since the existing MMBench evaluations are optimized for standard questions, directly using them would assign standard options to refusal responses. Therefore, we made the following modifications for the UPD challenge.
+![](images/8527d9d103d79fb90dfe083e26ab1afab0d0e32e3aaff53a8cc8710241fbd81d.jpg)  
+Figure A: Relationship between OC-Dual accuracy and Dual accuracy.
+Simplification of the Matching Algorithm. To apply the matching algorithm for UPD, we simplify the matching algorithm to prevent the refusal responses from matching the given options. In detail, when an option is denoted simply by a letter such as ‘A’ or expressed as ‘A) XXX’, ‘A. XXX’, ‘A, XXX’, ‘(A) XXX’ without the inclusion of other choices within the ‘XXX’ portion, it is considered that ‘A’ is being predicted.
+Change of the Template for GPT Evaluation. Next, to identify the refusal prediction, we leverage GPT following MMBench. We leverage GPT-4omini (gpt-4o-mini-2024-07-18), considering its high performance and low cost.
+We slightly change the template for the original MMBench, and create the query template for each setting in Fig. D. As for \${option}, we add UPDspecific options to recognize UPD predictions. In Fig. E, we illustrate the options for each setting. For AAD, we add two options: a masked correct option, and the option of “The correct answer is No answer, None of the above, all provided options are incorrect, or I cannot answer.”. For IASD, we add two options: a masked correct option, and the option of “The correct answer is No answer, None of the above, all provided options are irrelevant or incorrect, or I cannot answer.”. For IVQD, we add an option of “The correct answer is that The image is incompatible with the question, or I cannot answer.” For the additional-instruction setting, we also add the option “F. None of the above” or “F. The image and question are irrelevant.”. In each setting, we regard the options indicated by check marks (Fig. E), as correct ones.
+## E.3 Comparison to Human Decision
+In Fig. F, we investigate the alignment of scores given by GPT-4o-mini and humans for the base setting. To investigate the performance of the UPD predictions, we sampled every 100 predictions of LLaVA-Next-34B and GPT-4o output that were not matched by pattern matching and manually evaluated them. We found that the match rate with human evaluations is sufficiently high.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+F1: Different Performance Trends of MM-Bench and MM-UPD Bench. Table 1 shows that the performance trends of MMBench (Orig) and MM-UPD (Base/Opt/Inst) are completely different. For instance, although LLaVA-OV-7B (Li et al., 2024a), CogVLM2 (Hong et al., 2024), and Xgen-MM (Xue et al., 2024) exhibit very high performance (&gt;80%) in all Original Standard, their performances in the UPD Base setting drop to less than 6% in all Base settings. To investigate the correlation more rigorously, we calculate the correlation coefficients between the Original Standard and Dual accuracy/UPD accuracy in Table 2. We found that the correlation coefficient between UPD accuracy and the Original Standard is quite low (Max: 39.1, Min: 6.5). Dual accuracies still do not indicate a strong correlation. This suggests that our benchmark is capable of accurately capturing an important aspect of trustworthiness that has not been measured by previous benchmarks.
+F2: Large Gap between Open-source LMMs and Closed-source LMMs. As shown in Table 1, there is a significant performance gap between open-source LMMs and closed-source LMMs. One of the reasons for this performance gap is the training difference: Closed-source models are trained for refusal considering real-world user applications according to their system cards (Hurst et al., 2024; OpenAI, 2023). On the other hand, open-source models usually compete for performance with limited publicly available benchmarks. However, among open-source LMMs, models with large LLMs such as LLaVA-NeXT-34B and
+InternVL2-40B demonstrate performance comparable to closed-source models. Compared to smaller models trained on the same VQA data, such as LLaVA-NeXT-13B and InternVL2-2B/8B, there is a significant performance improvement, suggesting that the performance of the base LLM also plays a crucial role. However, a detailed check of each output reveals that a quality gap still exists between these powerful open-source LMMs and closed-source LMMs (refer to Appendix F.2).
+Next, we provide detailed findings below to support the rationale behind the above findings.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Assessing the understanding capability of LMMs is crucial for advancing fundamental progress. Multiple-Choice Question Answering (MCQA) serves as a fundamental format for understanding evaluation and is widely used in wellestablished benchmarks such as MMBench (Liu et al., 2024e) and MMMU (Yue et al., 2024a). Each MCQA instance consists of a question paired with multiple answer options, requiring models to select the correct one. MCQA enables precise evaluation of LMMs and facilitates solid progress in the field. Consequently, many MCQA-based benchmarks have been proposed recently (Fu et al., 2024; Yue et al., 2024b; Hu et al., 2025).
+Despite the advanced performance of LMMs on the accuracy of MCQA-format benchmarks, concerns remain regarding the reliability of their predictions. While previous works in the field of LLMs have discussed challenges such as maintaining invariance to different orderings of answer choices (Robinson et al., 2023; Wang et al., 2024a; Zheng et al., 2025), overcoming order sensitivity alone is not sufficient to ensure that the model truly understands the correct answer. A more recent study (Wang et al., 2025) investigated LLMs’ ability to reject unsolvable problems, such as questions where the correct answer is not present among the given choices. The ability to reject unsolvable problems can serve as a more reliable means of verifying the model’s true understanding. However, this study does not focus on LMMs. When extending the evaluation from LLMs to LMMs, the types of unsolvable problems differ. Additionally, there is a lack of benchmarks and systematic evaluation protocols for comprehensively assessing recent LMMs. Consequently, existing works fail to assess the depth of LMMs’ robust comprehension.
+To assess the robust comprehension of LMMs, we propose Unsolvable Problem Detection (UPD), which examines the LMM’s ability to withhold answers when faced with unsolvable problems. UPD encompasses three distinct settings: Absent Answer Detection (AAD), Incompatible Answer Set Detection (IASD), and Incompatible Visual Question Detection (IVQD). Fig. 1 shows the illustration of each setting. AAD evaluates whether the model declines to provide an answer when the correct answer is absent. IASD examines whether the model rejects a question when the given answer set is entirely incompatible. IVQD investigates the model’s ability to reject a question when there is no relevance between the image and the text question. A model that effectively rejects unsolvable problems while accurately solving standard solvable problems can be regarded as truly understanding them. On the other hand, a model that incorrectly selects an answer for unsolvable problems cannot be considered to have a true understanding of them.
+For the evaluation, we introduce MM-UPD Bench, a carefully designed benchmark for evaluating UPD capability across various ability dimensions. MM-UPD employs a rigorous three-step construction process that builds upon MMBench (Liu et al., 2024e): (1) filtering out questions that can be answered by text-only language models, (2) applying the carefully designed approach for creating UPD questions, (3) finally, manually removing ambiguous samples. Built on the foundation of MMBench, our benchmarks allow us to highlight the difficulty of MM-UPD by comparing it to the self-established MMBench, and also serves as a fine-grained diagnostic tool, offering detailed insights into each LMM’s weaknesses in a broad range of MMBench’s abilities.
+Our experimental results demonstrate the difficulty of MM-UPD across various state-of-the-art LMMs. The most important finding is that there is little correlation between the performance on the existing MMBench and MM-UPD Bench. This indicates that the community’s efforts to improve performance on existing benchmarks do not directly contribute to enhancing model reliability. In particular, we found that the gap between open-source and closed-source models is large, while opensource LMMs outperform closed-source LMMs on MMBench. Furthermore, our fine-grained ability analysis revealed that even closed-source models such as GPT-4o (Hurst et al., 2024) exhibit weaknesses in specific abilities.
+Finally, we revealed that whether the bottleneck lies in the LLM’s refusal capability or its visual understanding depends on the specific LMM. For LMMs where the bottleneck is in the LLM’s refusal capability, we observed performance improvements with LLM-driven approaches such as chain-of-thought (Kojima et al., 2022) and selfreflection (Kadavath et al., 2022).
+Our contributions are summarized as follows:
+• Definition of Unsolvable Problem Detection: We propose a novel challenge called Unsolvable Problem Detection, which evaluates the LMM’s robust understanding in three problem settings: AAD, IASD, and IVQD.
+• Construction of MM-UPD Bench: We rigorously construct the MM-UPD Bench and provide a fine-grained diagnostic tool for broader abilities.
+• Benchmarking with Recent LMMs: We evaluate state-of-the-art LMMs on the UPD problem and show that our benchmarks represent a new and meaningful dimension of the performances of LMMs.
+## 2 Related Work
+Vulnerability of MCQA Evaluation. The vulnerability of MCQA has mainly been researched in the field of LLM. Previous work has aimed to mitigate bias in answer options and enhance LLMs’ consistency across different option orders (Robinson et al., 2023; Wang et al., 2024a; Zheng et al., 2025). As a more recent work, Wang et al. (2025) tested LLM’s ability to refuse unsolvable problems. They found that LLMs may perform MCQA by selecting the least incorrect option rather than distinctly correct. However, it only deals with AAD, and when applied to LMMs, the types of unsolvable problems are limited. Additionally, we consider that handling unsolvable problems requires rigorous evaluation based on ability-specific assessments, while they have not clearly identified the performance differences across abilities.
+Unsolvable Problems. Unsolvable questions have been studied in NLP (Rajpurkar et al., 2018; Choi et al., 2018; Reddy et al., 2019; Sulem et al., 2022) and in VQA before the rise of LMMs (Gurari et al., 2018; Bhattacharya et al., 2019; Davis, 2020; Whitehead et al., 2022). Early VQA studies focused on task-specific models, making their benchmarks misaligned with modern LMMs due to task simplicity or differing evaluation protocols. While recent works have explored unsolvable questions in LMMs (Guo et al., 2024; Akter et al., 2024; Cao et al., 2024), they do not assess the robustness of LMMs for common MCQA.
+Answer Refusal. In the task of refusing to provide an answer, there are studies in the field of LLMs that focus on abstaining due to a lack of knowledge (Kadavath et al., 2022; Feng et al., 2024). The main difference between their work and ours is that while they focus on knowledge gaps, we focus on the flaws or incompleteness of the problem itself, which leads to a different problem formulation.
+## 3 Problem Definition
+In this section, we introduce the concept of Unsolvable Problem Detection (UPD), a task designed to evaluate models’ capacity to not blindly offer incorrect answers when presented with unsolvable problems. We consider various discrepancies among the provided image, question, and answer options.
+Then, we categorize UPD into three distinct problem types: Absent Answer Detection (AAD), Incompatible Answer Set Detection (IASD), and Incompatible Visual Question Detection (IVQD). Here, AAD has been proposed as an unsolvable type for LLMs in existing work (Wang et al., 2025), but it has not been examined with LMMs. Additionally, by incorporating IASD and IVQD, we can cover a broader scope of unsolvable types, enabling a more precise diagnosis of model weaknesses. The details of each setting are as follows:
+1. Absent Answer Detection (AAD): AAD tests the model’s capability to recognize when the correct answer is absent from the provided choices. It challenges the model to not only analyze the content of questions and images but also identify when it cannot select a correct response due to the absence of an appropriate option.
+2. Incompatible Answer Set Detection (IASD): IASD tests the model’s ability to identify situations where the set of answer choices is incompatible with the context. Differing from AAD, in which the answer set is related to the question or the image, IASD deals with answer sets that are entirely irrelevant, challenging the model to withhold a response due to the lack of reasonable options. By giving a completely unrelated answer set, IASD evaluates the inherent capacity of LMMs to withhold answering, which is not affected by the granularity of the given choices.
+3. Incompatible Visual Question Detection (IVQD): IVQD evaluates the LMMs’ capability to discern when a question and image are irrelevant or inappropriate. This setting tests the model’s understanding of the alignment between visual content and textual questions, aiming to spot instances where image-question pairs are incompatible.
+## 4 Benchmarks and Evaluations
+## 4.1 Construction of MM-UPD Bench
+We create MM-UPD Bench based on MMBench (dev, 20231003) (Liu et al., 2024e). MM-Bench (Liu et al., 2024e) is a systematically designed benchmark for evaluating various abilities of LMMs. Utilizing MMBench allows us to assess the reliability of LMMs for general VQA questions and also enables fine-grained, ability-wise evaluation (e.g., , “Coarse Perception: Image Scene” and “Logic Reasoning: Future Prediction”).
+To create MM-UPD Bench, we first filter imageagnostic questions from MMBench.
+![](images/8e55325c0797874808fbf88e4726d2818c53ea647ec576f6895753b97614baa6.jpg)  
+Figure 2: Examples of standard and UPD questions in each scenario. We evaluate all 4 four scenarios (Standard, AAD, IASD, and IVQD) as follows: the base setting, where no UPD-specific options/instructions are provided; the Option setting, which includes an option like “None of the above"; and the Instruction setting, where explicit guidance such as “Answer F. None of the above" is given. We calculate the Dual accuracy with the prediction of each Standard-UPD question pair (e.g., Standard-base and AAD-base).
+Filtering Image-Agnostic Questions. Most existing benchmarks, including MMBench, contain some image-agnostic questions (Chen et al., 2024b), which can be answered with only text information. This hinders the accurate evaluation of LMM performance. To address this issue, we first removed image-agnostic questions with text-only GPT-4 (Achiam et al., 2023). To eliminate the effect of random guessing, we applied CircularEval, which is explained in Sec. 4.4, for filtering. Next, we carefully examined the extracted question to guarantee neglectable impact of GPT-4 bias. After that, we manually eliminated the few remaining image-agnostic questions.
+Next, we will construct MM-AAD, MM-IASD, and MM-IVQD, which constitute MM-UPD.
+1. MM-AAD Bench: MM-AAD Bench is a dataset where the correct answer option for each question is removed. When creating the MM-AAD Bench, we mask the correct options and remove all questions that originally have two options (which after removal would have only one option left). To ensure no answer is present in the options, we also manually remove some questions with ambiguity. Our MM-AAD Bench has 820 AAD questions over 18 abilities.
+2. MM-IASD Bench: MM-IASD Bench is a dataset where the answer set is completely incompatible with the context specified by the question and the image. To create MM-IASD, we shuffle all questions and answer sets and pair each question with a random answer set. To further ensure the incompatibility, after the shuffling, we manually removed questions where the shuffled answer set was somehow compatible with the question. Our MM-IASD Bench has 919 IASD questions over 18 abilities.
+3. MM-IVQD Bench: MM-IVQD Bench is a dataset where the image and question are incompatible. This is achieved by focusing on questions that are specific, which are more likely to be incompatible with a randomly picked image. Specifically, we first exclude the questions that can be relevant to most images (e.g., , “Which one is the correct caption of this image?”) and then shuffle the original image-question pairs. Again, we conduct a manual check to guarantee the incompatibility of image-question pairs. Our MM-IVQD Bench has 356 IVQD questions over 12 abilities.
+In total, our UPD benchmark consists of 2,095 questions. Note here that although the MM-UPD Bench utilizes source data from MMBench, our construction approach enables us to emphasize the difficulty of MM-UPD by comparing the performance to the established MMBench, providing a deeper insight than creating an entirely new benchmark. Here, we also considered adopting MMMU (Yue et al., 2024a). However, preliminary experiments showed that due to MMMU’s high difficulty level, the accuracy for standard questions was still low, making it challenging to assess reliability and potentially causing critical insights to be overlooked (as discussed in Appendix B.6). More detailed information for the construction process is provided in Appendix B.
+## 4.2 Evaluation Metrics
+To capture the ideal behavior of LMMs, we define several metrics and evaluate their performance under both standard and UPD settings. Ideal LMMs should not only yield correct answers in the standard setting (where the image, question, and answer sets are all aligned and the ground-truth answer is always within the options) but also be able to withhold answering in the UPD scenario where the question becomes unsolvable. In Fig. 2, we show the examples of these standard and UPD settings. Here, for AAD, the standard scenario refers to the correct answer included in the provided answer set. For IASD, the standard scenario refers to the correct answer included in the provided answer set and the rest options are also relevant. For IVQD, given the same question and answer set, the standard scenario has a compatible image. To better reflect the ideal behavior of LMMs, we measure several metrics throughout the paper:
+1. Standard Accuracy: The accuracy on standard questions in Fig. 2.
+2. UPD (AAD/IASD/IVQD) Accuracy: The accuracy of AAD/IASD/IVQD questions in Fig. 2 (AAD/IASD/IVQD).
+3. Dual Accuracy: The accuracy on standard-UPD pairs, where we count success only if the model is correct on both the standard and UPD questions. This metric considers both Standard and UPD performances, making it the most suitable evaluation metric for UPD. Our evaluation thus uses this as the primary metric.
+4. Original Standard: This refers to the Standard accuracy evaluated using the prompt for the original MMBench. By adding the prompt “Answer with the option’s letter from the given choices directly" at the end of the question, it focuses specifically on improving Standard accuracy performance at the expense of UPD performance. While the Original Standard score is not Dual accuracy, we consider it the upper bound of Dual accuracy for each model based on the definition of Dual accuracy.
+## 4.3 Evaluation Setting
+To reflect the real-world use cases, we test in three settings, including a basic one and two carefully designed ones that attempt to address UPD with prompt engineering.
+1. Base Setting: In the base setting, no instructions and options are provided to the model to withhold answers (shown in Fig. 2 (a)). This setting represents the most common case for using LMMs in the real world.
+2. Option Setting: We add extra option “None of the above” for AAD and IASD and “The image and question are irrelevant.” for IVQD, respectively (shown in Fig. 2 (b)). Following LLaVA (Liu et al., 2024c), we also add an instruction of “Answer with the option’s letter from the given choices directly.” to reinforce the instruction following capability.
+3. Instruction Setting: We add additional instruction to explicitly gear the model towards acknowledging the unsolvable problem. The instruction is “If all the options are incorrect, answer F. None of the above.” for AAD and IASD and “If the given image is irrelevant to the question, answer F. The image and question are irrelevant.” for IVQD, respectively.
+Note here that these additional options and instructions are also added to the questions in standard scenarios to make a fair comparison.
+## 4.4 Evaluation Protocol
+We adopt Circular Evaluation and GPT-involved Choice Extraction in MMBench (Liu et al., 2024e). In Circular Evaluation, a problem is tested multiple times with circularly shifted choices, and the LMM needs to succeed in all tests to pass. GPT-involved Choice Extraction first performs the matching algorithm and then uses GPT for those that do not match. To accurately identify when the model predicts as “no answer”, we leverage GPT-4omini (gpt-4o-mini-2024-07-18). Specifically, we count as correct for UPD questions if the model’s output is similar to “none of the above”, “I cannot answer”, or the masked correct option for AAD and IASD and “the image is irrelevant” or “I cannot answer” for IVQD. The details are shown in Appendix E.2.
+## 5 Experiments
+## 5.1 Experimental Setups
+We evaluated the performance of open-source and closed-source LMMs from lightweight models to 40B models. For inference, we perform a greedy search for all LMMs.
+</t>
+  </si>
+  <si>
+    <t>The chunk references MM‑UPD Bench but only shows a mapping table; it does not explain what MM‑UPD Bench stands for.</t>
+  </si>
+  <si>
     <t>The chunk explicitly describes that when refining problems, annotators record detailed justifications in comments, discuss disagreements, and reach consensus, directly addressing the query about the need for detailed justification during curation.</t>
   </si>
   <si>
     <t>The chunk discusses Dual accuracy but does not mention OC‑Dual accuracy or any correlation between the two metrics, so it only loosely relates to the query.</t>
   </si>
   <si>
-    <t>The chunk explicitly states that self‑reflection enables models to judge and evaluate their own answers, directly answering the query.</t>
+    <t>The chunk discusses self‑reflection as a method for models to evaluate their own responses, indicating preliminary capabilities for judging answers. It partially addresses the query but does not fully elaborate on effectiveness or limitations.</t>
   </si>
   <si>
     <t>The chunk contains a bibliography of AI research papers and does not mention ropes, harnesses, cliff faces, or any climbing activity. It is completely unrelated to the query.</t>
   </si>
   <si>
-    <t>Yes – when a problem is refined during curation, the reason must be recorded in detail as a comment, ensuring a clear justification for the change.</t>
-  </si>
-  <si>
-    <t>Yes – the text explains that self‑reflection lets the model look at its own output, and prior work has shown that LLMs can preliminarily judge and evaluate their answers.</t>
-  </si>
-  <si>
-    <t>The answer directly confirms that detailed justification is required and cites the same practice described in the retrieved chunk, fully addressing the query.</t>
-  </si>
-  <si>
-    <t>The answer does not address the question about the correlation between OC-Dual accuracy and Dual accuracy.</t>
-  </si>
-  <si>
-    <t>The answer directly confirms that self‑reflection enables models to evaluate their own answers, matching the retrieved text that states LLMs can judge and evaluate their responses.</t>
-  </si>
-  <si>
-    <t>The answer correctly identifies rock climbing as the activity that uses ropes and harnesses on a cliff face, fully addressing the user’s question. However, the retrieved chunk is irrelevant (relevancy score 0), so grounding cannot be assessed.</t>
+    <t>The chunk mentions Dual accuracy and presents comparison results, but it does not explain why Dual accuracy is considered effective for assessing LMM reliability.</t>
+  </si>
+  <si>
+    <t>The chunk explicitly defines UPD as a task to evaluate LMMs’ ability to recognize and withhold answers for unsolvable MCQA problems, directly answering the query about its purpose.</t>
+  </si>
+  <si>
+    <t>The chunk discusses UPD instruction tuning, shows that UPD-specific training improves UPD performance but can degrade general task performance, directly addressing the query.</t>
+  </si>
+  <si>
+    <t>The chunk discusses a performance gap between open‑source and closed‑source LMMs, indicating closed‑source models generally perform better, but also notes that some large open‑source models approach that performance. It partially answers the query but does not fully quantify or conclude definitively.</t>
+  </si>
+  <si>
+    <t>The chunk explains UPD as a task where LMMs must refuse unsolvable MCQA problems (AAD, IASD, IVQD), contrasting it with standard MCQA that only requires selecting a correct answer. It details the differences, benchmark construction, and evaluation metrics, directly answering how UPD differs from traditional MCQA.</t>
+  </si>
+  <si>
+    <t>Yes – annotators must record a detailed justification (e.g., a comment explaining why an image relates to a question or why changing it would create irrelevance). If another annotator agrees, the refinement proceeds; if not, all four discuss until consensus is reached.</t>
+  </si>
+  <si>
+    <t>Yes – the paper notes that self‑reflection “has been shown that LLMs might have preliminary capabilities for judging and evaluating their own answers” and the authors evaluate this ability in their experiments.</t>
+  </si>
+  <si>
+    <t>Dual accuracy is effective because it directly measures how far a model’s performance is from the best‑possible (Upper Bound) performance. The clear gap between each model’s Dual accuracy and the Original Standard value shows exactly how much lower the open‑source LMMs perform, giving a concise, quantifiable assessment of their reliability.</t>
+  </si>
+  <si>
+    <t>Unsolvable Problem Detection (UPD) is a task that tests whether a Large Multimodal Model can recognize when a multiple‑choice question cannot be answered—because the answer is missing, the answer options are contradictory, or the image does not match the question—and correctly withhold a response. In this way, UPD evaluates a model’s robust understanding and trustworthiness beyond its ability to pick a correct answer.</t>
+  </si>
+  <si>
+    <t>Yes. The text notes that while UPD‑specific instruction tuning improves UPD accuracy, it can **degrade performance on other general tasks**.</t>
+  </si>
+  <si>
+    <t>Yes. The evaluation shows a clear performance gap in favor of closed‑source LMMs. While large open‑source models (e.g., LLaVA‑NeXT‑34B, InternVL2‑40B) can approach closed‑source performance, a detailed check still reveals a quality gap, indicating that closed‑source models tend to offer better responses.</t>
+  </si>
+  <si>
+    <t>UPD turns the usual MCQA task on its head by adding **unsolvable problem settings** that a model must recognize and *refuse* to answer.  
+While standard MCQA simply asks the LMM to pick the right option from a list that always contains the correct answer, UPD introduces three new scenarios:
+| Setting | What the model faces |
+|---------|---------------------|
+| **AAD** | The correct answer is **absent** from the choice set. |
+| **IASD** | The entire answer set is **incompatible** with the question and image. |
+| **IVQD** | The image and the question are **incompatible**. |
+Thus, UPD measures a model’s *robustness* and *reliability*—whether it can withhold an answer when no valid option exists—rather than just its ability to pick the right choice. The evaluation also uses “dual accuracy,” requiring correct answers on both standard and UPD pairs, highlighting failures that pure MCQA accuracy would miss.</t>
+  </si>
+  <si>
+    <t>The answer does not provide the expansion of MM‑UPD Bench and therefore fails to address the user’s question.</t>
+  </si>
+  <si>
+    <t>The answer correctly states that detailed justification is required for refining problems and describes the consensus process, matching the retrieved chunk’s description of recording detailed comments and reaching agreement among annotators.</t>
+  </si>
+  <si>
+    <t>The answer does not address the user’s question about the correlation between OC-Dual accuracy and Dual accuracy.</t>
+  </si>
+  <si>
+    <t>The answer directly confirms that self‑reflection enables models to evaluate their own answers, matching the query. It aligns with the retrieved chunk, which states that LLMs have preliminary capabilities for judging and evaluating their responses. Thus, it fully addresses the question and is faithful to the context.</t>
+  </si>
+  <si>
+    <t>The answer does not provide any information about an activity involving ropes and harnesses on a cliff face, so it fails to address the user’s question.</t>
+  </si>
+  <si>
+    <t>The answer explains that Dual accuracy measures how far a model is from the upper bound and provides a quantifiable reliability metric, directly addressing the question. Retrieval relevance is low, so grounding cannot be evaluated.</t>
+  </si>
+  <si>
+    <t>The answer accurately explains UPD’s purpose—detecting unsolvable MCQA cases and testing a model’s ability to withhold answers—matching the retrieved description. It is fully consistent with the source.</t>
+  </si>
+  <si>
+    <t>The answer directly states that UPD‑specific training can degrade general task performance, which fully answers the query. The retrieved chunk explicitly mentions the same effect, so the answer is consistent with the context.</t>
+  </si>
+  <si>
+    <t>The answer directly states that closed‑source models outperform open‑source ones, matching the retrieved chunk that reports a significant performance gap favoring closed‑source LMMs. It fully addresses the user’s question and is consistent with the evidence.</t>
+  </si>
+  <si>
+    <t>The answer fully explains that UPD focuses on detecting unsolvable problems (AAD, IASD, IVQD) and contrasts this with standard MCQA, which always has a correct option. It aligns with the retrieved chunk and is consistent with the context.</t>
   </si>
 </sst>
 </file>
@@ -711,7 +1047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -766,43 +1102,40 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="H2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M2">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2">
-        <v>3</v>
-      </c>
-      <c r="K2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M2">
-        <v>3</v>
-      </c>
-      <c r="N2" t="b">
-        <v>1</v>
-      </c>
       <c r="O2" t="s">
-        <v>44</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -810,43 +1143,43 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="I3" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K3" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
       </c>
       <c r="O3" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -854,46 +1187,43 @@
         <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="I4" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="L4" t="s">
         <v>43</v>
       </c>
       <c r="M4">
-        <v>3</v>
-      </c>
-      <c r="N4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -901,43 +1231,322 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" t="s">
+        <v>63</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>72</v>
+      </c>
+      <c r="L5" t="s">
+        <v>80</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="s">
+        <v>54</v>
+      </c>
+      <c r="I6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="O6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" t="s">
+        <v>62</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L7" t="s">
+        <v>81</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
+      </c>
+      <c r="O7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" t="s">
         <v>21</v>
       </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="B8" t="s">
         <v>25</v>
       </c>
-      <c r="E5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
-      </c>
-      <c r="I5" t="s">
-        <v>37</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8">
+        <v>3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L8" t="s">
+        <v>82</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" t="s">
+        <v>66</v>
+      </c>
+      <c r="J9">
+        <v>3</v>
+      </c>
+      <c r="K9" t="s">
+        <v>76</v>
+      </c>
+      <c r="L9" t="s">
+        <v>83</v>
+      </c>
+      <c r="M9">
+        <v>3</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>58</v>
+      </c>
+      <c r="I10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
+      <c r="K10" t="s">
+        <v>77</v>
+      </c>
+      <c r="L10" t="s">
+        <v>84</v>
+      </c>
+      <c r="M10">
+        <v>3</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
         <v>41</v>
       </c>
-      <c r="L5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5">
-        <v>3</v>
-      </c>
-      <c r="O5" t="s">
-        <v>47</v>
+      <c r="E11" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>59</v>
+      </c>
+      <c r="I11" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11">
+        <v>3</v>
+      </c>
+      <c r="K11" t="s">
+        <v>78</v>
+      </c>
+      <c r="L11" t="s">
+        <v>85</v>
+      </c>
+      <c r="M11">
+        <v>3</v>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>